<commit_message>
Update  infiltration rate table for some pototypes
</commit_message>
<xml_diff>
--- a/Specifications/Nonresidential/v2.0/RetailStripMall_Prototype_Scorecard.xlsx
+++ b/Specifications/Nonresidential/v2.0/RetailStripMall_Prototype_Scorecard.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cursor\Check dictation and Spelling\Clean-uploaded to GH-6Oct2026\Without Weights\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\NOR-Codes-Stds\CalBEM-Prototypes\Specifications\Nonresidential\v2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D5482A-03AE-49FF-BFCC-CB8EFB9FC8EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED9C33D8-D13F-4486-9487-69DD60FC19EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="890" firstSheet="1" activeTab="1" xr2:uid="{EAC23EE3-0CA0-4FF8-990D-9B21A59FA3E0}"/>
   </bookViews>
@@ -983,6 +983,7 @@
         <sz val="12"/>
         <color rgb="FFFFFFFF"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Efficiency of HVAC System
 </t>
@@ -992,6 +993,7 @@
         <sz val="10"/>
         <color rgb="FFFFFFFF"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> (Efficiency is capacity-dependent. The following table provides a general estimate of system efficiency based on preliminary simulations in one climate zone, or assuming cooling load based on rule of thumb)</t>
     </r>
@@ -2421,11 +2423,13 @@
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="55">
@@ -2738,7 +2742,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="185">
+  <borders count="190">
     <border>
       <left/>
       <right/>
@@ -5066,6 +5070,67 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -5135,7 +5200,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="601">
+  <cellXfs count="604">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -6357,6 +6422,9 @@
     <xf numFmtId="0" fontId="13" fillId="9" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6366,9 +6434,6 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6396,50 +6461,56 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6447,9 +6518,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="178" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6471,15 +6539,9 @@
     <xf numFmtId="0" fontId="45" fillId="41" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="5" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="54" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6489,12 +6551,6 @@
     <xf numFmtId="0" fontId="59" fillId="9" borderId="162" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6603,6 +6659,144 @@
     <xf numFmtId="0" fontId="13" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="108" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="107" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="102" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="103" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="104" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="87" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="87" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="79" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="80" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="88" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="89" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="148" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6633,54 +6827,12 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="140" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="103" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="141" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="80" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6690,15 +6842,6 @@
     <xf numFmtId="0" fontId="51" fillId="0" borderId="81" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="79" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="80" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6708,93 +6851,6 @@
     <xf numFmtId="0" fontId="50" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="88" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="89" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="87" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="108" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="107" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="102" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="104" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="87" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6836,6 +6892,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="186" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="187" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="188" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="185" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="189" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="175" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="66">
@@ -15987,14 +16061,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="441" t="s">
+      <c r="A1" s="442" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="441"/>
-      <c r="C1" s="441"/>
+      <c r="B1" s="442"/>
+      <c r="C1" s="442"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="442" t="s">
+      <c r="A2" s="443" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -16003,7 +16077,7 @@
       <c r="C2" s="316"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="442"/>
+      <c r="A3" s="443"/>
       <c r="B3" s="348" t="s">
         <v>3</v>
       </c>
@@ -16015,7 +16089,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="442"/>
+      <c r="A4" s="443"/>
       <c r="B4" s="348" t="s">
         <v>6</v>
       </c>
@@ -16027,7 +16101,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="442"/>
+      <c r="A5" s="443"/>
       <c r="B5" s="6" t="s">
         <v>8</v>
       </c>
@@ -16039,7 +16113,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="442" t="s">
+      <c r="A6" s="443" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -16053,7 +16127,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="442"/>
+      <c r="A7" s="443"/>
       <c r="B7" s="3" t="s">
         <v>13</v>
       </c>
@@ -16065,7 +16139,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="442"/>
+      <c r="A8" s="443"/>
       <c r="B8" s="3" t="s">
         <v>15</v>
       </c>
@@ -16077,17 +16151,17 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="442"/>
+      <c r="A9" s="443"/>
       <c r="C9" s="127"/>
       <c r="D9" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A10" s="442" t="s">
+      <c r="A10" s="443" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="443" t="s">
+      <c r="B10" s="444" t="s">
         <v>18</v>
       </c>
       <c r="C10" s="275" t="s">
@@ -16098,8 +16172,8 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="442"/>
-      <c r="B11" s="443"/>
+      <c r="A11" s="443"/>
+      <c r="B11" s="444"/>
       <c r="C11" s="275" t="s">
         <v>20</v>
       </c>
@@ -16108,7 +16182,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="442"/>
+      <c r="A12" s="443"/>
       <c r="B12" s="350" t="s">
         <v>22</v>
       </c>
@@ -16120,7 +16194,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="442"/>
+      <c r="A13" s="443"/>
       <c r="B13" s="276" t="s">
         <v>24</v>
       </c>
@@ -16132,7 +16206,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="442"/>
+      <c r="A14" s="443"/>
       <c r="B14" s="350" t="s">
         <v>26</v>
       </c>
@@ -16144,7 +16218,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="442" t="s">
+      <c r="A15" s="443" t="s">
         <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -16158,7 +16232,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="442"/>
+      <c r="A16" s="443"/>
       <c r="B16" s="348" t="s">
         <v>31</v>
       </c>
@@ -16170,7 +16244,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="442"/>
+      <c r="A17" s="443"/>
       <c r="B17" s="6" t="s">
         <v>33</v>
       </c>
@@ -16182,7 +16256,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="442"/>
+      <c r="A18" s="443"/>
       <c r="B18" s="90" t="s">
         <v>34</v>
       </c>
@@ -16194,7 +16268,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="442"/>
+      <c r="A19" s="443"/>
       <c r="B19" s="3" t="s">
         <v>36</v>
       </c>
@@ -16206,7 +16280,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="442"/>
+      <c r="A20" s="443"/>
       <c r="B20" s="350" t="s">
         <v>38</v>
       </c>
@@ -16218,7 +16292,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="442"/>
+      <c r="A21" s="443"/>
       <c r="B21" s="6" t="s">
         <v>40</v>
       </c>
@@ -16230,7 +16304,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A22" s="442"/>
+      <c r="A22" s="443"/>
       <c r="B22" s="351" t="s">
         <v>42</v>
       </c>
@@ -16242,7 +16316,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="25.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="442"/>
+      <c r="A23" s="443"/>
       <c r="B23" s="7" t="s">
         <v>44</v>
       </c>
@@ -16254,7 +16328,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="442"/>
+      <c r="A24" s="443"/>
       <c r="B24" s="352" t="s">
         <v>46</v>
       </c>
@@ -16266,7 +16340,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="442"/>
+      <c r="A25" s="443"/>
       <c r="B25" s="352" t="s">
         <v>48</v>
       </c>
@@ -16278,7 +16352,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="442"/>
+      <c r="A26" s="443"/>
       <c r="B26" s="352" t="s">
         <v>50</v>
       </c>
@@ -16290,48 +16364,48 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="442"/>
+      <c r="A27" s="443"/>
       <c r="C27" s="262"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C28" s="316"/>
     </row>
     <row r="29" spans="1:4" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A29" s="441" t="s">
+      <c r="A29" s="442" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="441"/>
-      <c r="C29" s="441"/>
+      <c r="B29" s="442"/>
+      <c r="C29" s="442"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="444" t="s">
+      <c r="A30" s="441" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="444"/>
-      <c r="C30" s="444"/>
+      <c r="B30" s="441"/>
+      <c r="C30" s="441"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="444"/>
-      <c r="B31" s="444"/>
-      <c r="C31" s="444"/>
+      <c r="A31" s="441"/>
+      <c r="B31" s="441"/>
+      <c r="C31" s="441"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="444"/>
-      <c r="B32" s="444"/>
-      <c r="C32" s="444"/>
+      <c r="A32" s="441"/>
+      <c r="B32" s="441"/>
+      <c r="C32" s="441"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="B10:B11"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="A30:C30"/>
     <mergeCell ref="A15:A27"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A14"/>
-    <mergeCell ref="B10:B11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C23" r:id="rId1" xr:uid="{615EECC0-DAAB-4A87-8792-2805AA13E96C}"/>
@@ -16381,13 +16455,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="516" t="str">
+      <c r="A1" s="513" t="str">
         <f>"Exterior Lighting - "&amp;Prototype!A2</f>
         <v>Exterior Lighting - RetailStripMall</v>
       </c>
-      <c r="B1" s="516"/>
-      <c r="C1" s="516"/>
-      <c r="D1" s="516"/>
+      <c r="B1" s="513"/>
+      <c r="C1" s="513"/>
+      <c r="D1" s="513"/>
     </row>
     <row r="2" spans="1:8" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="35" t="s">
@@ -16431,24 +16505,24 @@
       <c r="C5" s="62"/>
     </row>
     <row r="6" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="516" t="s">
+      <c r="A6" s="513" t="s">
         <v>350</v>
       </c>
-      <c r="B6" s="516"/>
-      <c r="C6" s="516"/>
-      <c r="D6" s="516"/>
-      <c r="E6" s="516"/>
-      <c r="F6" s="516"/>
-      <c r="G6" s="516"/>
+      <c r="B6" s="513"/>
+      <c r="C6" s="513"/>
+      <c r="D6" s="513"/>
+      <c r="E6" s="513"/>
+      <c r="F6" s="513"/>
+      <c r="G6" s="513"/>
     </row>
     <row r="7" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="81" t="s">
         <v>351</v>
       </c>
-      <c r="B7" s="518" t="s">
+      <c r="B7" s="515" t="s">
         <v>352</v>
       </c>
-      <c r="C7" s="519"/>
+      <c r="C7" s="516"/>
       <c r="D7" s="123" t="s">
         <v>353</v>
       </c>
@@ -16607,42 +16681,42 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="517" t="s">
+      <c r="A14" s="514" t="s">
         <v>372</v>
       </c>
-      <c r="B14" s="517"/>
-      <c r="C14" s="517"/>
-      <c r="D14" s="517"/>
-      <c r="E14" s="517"/>
-      <c r="F14" s="517"/>
+      <c r="B14" s="514"/>
+      <c r="C14" s="514"/>
+      <c r="D14" s="514"/>
+      <c r="E14" s="514"/>
+      <c r="F14" s="514"/>
       <c r="G14" s="101">
         <f>SUM(G8:G13)-G15</f>
         <v>472.91529557599995</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="517" t="s">
+      <c r="A15" s="514" t="s">
         <v>373</v>
       </c>
-      <c r="B15" s="517"/>
-      <c r="C15" s="517"/>
-      <c r="D15" s="517"/>
-      <c r="E15" s="517"/>
-      <c r="F15" s="517"/>
+      <c r="B15" s="514"/>
+      <c r="C15" s="514"/>
+      <c r="D15" s="514"/>
+      <c r="E15" s="514"/>
+      <c r="F15" s="514"/>
       <c r="G15" s="101">
         <f>G11+G12</f>
         <v>346.56245453752001</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="517" t="s">
+      <c r="A16" s="514" t="s">
         <v>293</v>
       </c>
-      <c r="B16" s="517"/>
-      <c r="C16" s="517"/>
-      <c r="D16" s="517"/>
-      <c r="E16" s="517"/>
-      <c r="F16" s="517"/>
+      <c r="B16" s="514"/>
+      <c r="C16" s="514"/>
+      <c r="D16" s="514"/>
+      <c r="E16" s="514"/>
+      <c r="F16" s="514"/>
       <c r="G16" s="101">
         <f t="shared" ref="G16" si="0">G14+G15</f>
         <v>819.47775011351996</v>
@@ -16748,14 +16822,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="520" t="str">
+      <c r="A1" s="517" t="str">
         <f>"Equipment - "&amp;Prototype!A2</f>
         <v>Equipment - RetailStripMall</v>
       </c>
-      <c r="B1" s="521"/>
-      <c r="C1" s="521"/>
-      <c r="D1" s="521"/>
-      <c r="E1" s="522"/>
+      <c r="B1" s="518"/>
+      <c r="C1" s="518"/>
+      <c r="D1" s="518"/>
+      <c r="E1" s="519"/>
       <c r="F1" s="52"/>
     </row>
     <row r="2" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -16860,38 +16934,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="469" t="str">
+      <c r="A1" s="471" t="str">
         <f>"Schedules - "&amp;Prototype!A2</f>
         <v>Schedules - RetailStripMall</v>
       </c>
-      <c r="B1" s="469"/>
-      <c r="C1" s="469"/>
-      <c r="D1" s="469"/>
-      <c r="E1" s="469"/>
-      <c r="F1" s="469"/>
-      <c r="G1" s="469"/>
-      <c r="H1" s="469"/>
-      <c r="I1" s="469"/>
-      <c r="J1" s="469"/>
-      <c r="K1" s="469"/>
-      <c r="L1" s="469"/>
-      <c r="M1" s="469"/>
-      <c r="N1" s="469"/>
-      <c r="O1" s="469"/>
-      <c r="P1" s="469"/>
-      <c r="Q1" s="469"/>
-      <c r="R1" s="469"/>
-      <c r="S1" s="469"/>
-      <c r="T1" s="469"/>
-      <c r="U1" s="469"/>
-      <c r="V1" s="469"/>
-      <c r="W1" s="469"/>
-      <c r="X1" s="469"/>
-      <c r="Y1" s="469"/>
-      <c r="Z1" s="469"/>
-      <c r="AA1" s="469"/>
-      <c r="AB1" s="469"/>
-      <c r="AC1" s="566"/>
+      <c r="B1" s="471"/>
+      <c r="C1" s="471"/>
+      <c r="D1" s="471"/>
+      <c r="E1" s="471"/>
+      <c r="F1" s="471"/>
+      <c r="G1" s="471"/>
+      <c r="H1" s="471"/>
+      <c r="I1" s="471"/>
+      <c r="J1" s="471"/>
+      <c r="K1" s="471"/>
+      <c r="L1" s="471"/>
+      <c r="M1" s="471"/>
+      <c r="N1" s="471"/>
+      <c r="O1" s="471"/>
+      <c r="P1" s="471"/>
+      <c r="Q1" s="471"/>
+      <c r="R1" s="471"/>
+      <c r="S1" s="471"/>
+      <c r="T1" s="471"/>
+      <c r="U1" s="471"/>
+      <c r="V1" s="471"/>
+      <c r="W1" s="471"/>
+      <c r="X1" s="471"/>
+      <c r="Y1" s="471"/>
+      <c r="Z1" s="471"/>
+      <c r="AA1" s="471"/>
+      <c r="AB1" s="471"/>
+      <c r="AC1" s="548"/>
       <c r="AD1" s="39"/>
       <c r="AE1" s="39"/>
       <c r="AF1" s="39"/>
@@ -16902,47 +16976,47 @@
       <c r="AK1" s="40"/>
     </row>
     <row r="2" spans="1:39" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="535" t="s">
+      <c r="A2" s="546" t="s">
         <v>382</v>
       </c>
-      <c r="B2" s="535" t="s">
+      <c r="B2" s="546" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="535" t="s">
+      <c r="C2" s="546" t="s">
         <v>383</v>
       </c>
-      <c r="D2" s="535" t="s">
+      <c r="D2" s="546" t="s">
         <v>214</v>
       </c>
-      <c r="E2" s="535" t="s">
+      <c r="E2" s="546" t="s">
         <v>384</v>
       </c>
-      <c r="F2" s="558" t="s">
+      <c r="F2" s="563" t="s">
         <v>385</v>
       </c>
-      <c r="G2" s="558"/>
-      <c r="H2" s="558"/>
-      <c r="I2" s="558"/>
-      <c r="J2" s="558"/>
-      <c r="K2" s="558"/>
-      <c r="L2" s="558"/>
-      <c r="M2" s="558"/>
-      <c r="N2" s="558"/>
-      <c r="O2" s="558"/>
-      <c r="P2" s="558"/>
-      <c r="Q2" s="558"/>
-      <c r="R2" s="558"/>
-      <c r="S2" s="558"/>
-      <c r="T2" s="558"/>
-      <c r="U2" s="558"/>
-      <c r="V2" s="558"/>
-      <c r="W2" s="558"/>
-      <c r="X2" s="558"/>
-      <c r="Y2" s="558"/>
-      <c r="Z2" s="558"/>
-      <c r="AA2" s="558"/>
-      <c r="AB2" s="558"/>
-      <c r="AC2" s="558"/>
+      <c r="G2" s="563"/>
+      <c r="H2" s="563"/>
+      <c r="I2" s="563"/>
+      <c r="J2" s="563"/>
+      <c r="K2" s="563"/>
+      <c r="L2" s="563"/>
+      <c r="M2" s="563"/>
+      <c r="N2" s="563"/>
+      <c r="O2" s="563"/>
+      <c r="P2" s="563"/>
+      <c r="Q2" s="563"/>
+      <c r="R2" s="563"/>
+      <c r="S2" s="563"/>
+      <c r="T2" s="563"/>
+      <c r="U2" s="563"/>
+      <c r="V2" s="563"/>
+      <c r="W2" s="563"/>
+      <c r="X2" s="563"/>
+      <c r="Y2" s="563"/>
+      <c r="Z2" s="563"/>
+      <c r="AA2" s="563"/>
+      <c r="AB2" s="563"/>
+      <c r="AC2" s="563"/>
       <c r="AD2" s="39"/>
       <c r="AE2" s="39"/>
       <c r="AF2" s="39"/>
@@ -16953,11 +17027,11 @@
       <c r="AK2" s="40"/>
     </row>
     <row r="3" spans="1:39" ht="25.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="536"/>
-      <c r="B3" s="536"/>
-      <c r="C3" s="536"/>
-      <c r="D3" s="536"/>
-      <c r="E3" s="536"/>
+      <c r="A3" s="547"/>
+      <c r="B3" s="547"/>
+      <c r="C3" s="547"/>
+      <c r="D3" s="547"/>
+      <c r="E3" s="547"/>
       <c r="F3" s="325">
         <v>1</v>
       </c>
@@ -17040,16 +17114,16 @@
       <c r="AK3" s="40"/>
     </row>
     <row r="4" spans="1:39" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="552" t="s">
+      <c r="A4" s="549" t="s">
         <v>386</v>
       </c>
-      <c r="B4" s="556" t="s">
+      <c r="B4" s="582" t="s">
         <v>117</v>
       </c>
-      <c r="C4" s="540" t="s">
+      <c r="C4" s="565" t="s">
         <v>387</v>
       </c>
-      <c r="D4" s="559" t="s">
+      <c r="D4" s="564" t="s">
         <v>388</v>
       </c>
       <c r="E4" s="136" t="s">
@@ -17137,10 +17211,10 @@
       <c r="AK4" s="40"/>
     </row>
     <row r="5" spans="1:39" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="553"/>
-      <c r="B5" s="541"/>
-      <c r="C5" s="541"/>
-      <c r="D5" s="544"/>
+      <c r="A5" s="538"/>
+      <c r="B5" s="532"/>
+      <c r="C5" s="532"/>
+      <c r="D5" s="557"/>
       <c r="E5" s="139" t="s">
         <v>390</v>
       </c>
@@ -17226,10 +17300,10 @@
       <c r="AK5" s="40"/>
     </row>
     <row r="6" spans="1:39" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="567"/>
-      <c r="B6" s="542"/>
-      <c r="C6" s="542"/>
-      <c r="D6" s="545"/>
+      <c r="A6" s="539"/>
+      <c r="B6" s="541"/>
+      <c r="C6" s="541"/>
+      <c r="D6" s="558"/>
       <c r="E6" s="142" t="s">
         <v>391</v>
       </c>
@@ -17315,18 +17389,18 @@
       <c r="AK6" s="40"/>
     </row>
     <row r="7" spans="1:39" ht="38.700000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="552" t="str">
+      <c r="A7" s="549" t="str">
         <f>A4</f>
         <v>All Zones</v>
       </c>
-      <c r="B7" s="546" t="str">
+      <c r="B7" s="551" t="str">
         <f>B4</f>
         <v>Retail</v>
       </c>
-      <c r="C7" s="540" t="s">
+      <c r="C7" s="565" t="s">
         <v>392</v>
       </c>
-      <c r="D7" s="543" t="s">
+      <c r="D7" s="556" t="s">
         <v>393</v>
       </c>
       <c r="E7" s="145" t="s">
@@ -17415,10 +17489,10 @@
       <c r="AM7" s="51"/>
     </row>
     <row r="8" spans="1:39" ht="38.700000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="553"/>
-      <c r="B8" s="547"/>
-      <c r="C8" s="541"/>
-      <c r="D8" s="544"/>
+      <c r="A8" s="538"/>
+      <c r="B8" s="552"/>
+      <c r="C8" s="532"/>
+      <c r="D8" s="557"/>
       <c r="E8" s="148" t="s">
         <v>390</v>
       </c>
@@ -17505,10 +17579,10 @@
       <c r="AM8" s="51"/>
     </row>
     <row r="9" spans="1:39" ht="38.700000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="567"/>
-      <c r="B9" s="557"/>
-      <c r="C9" s="542"/>
-      <c r="D9" s="545"/>
+      <c r="A9" s="539"/>
+      <c r="B9" s="583"/>
+      <c r="C9" s="541"/>
+      <c r="D9" s="558"/>
       <c r="E9" s="151" t="s">
         <v>391</v>
       </c>
@@ -17595,18 +17669,18 @@
       <c r="AM9" s="51"/>
     </row>
     <row r="10" spans="1:39" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="552" t="str">
+      <c r="A10" s="549" t="str">
         <f>A4</f>
         <v>All Zones</v>
       </c>
-      <c r="B10" s="546" t="str">
+      <c r="B10" s="551" t="str">
         <f>B4</f>
         <v>Retail</v>
       </c>
-      <c r="C10" s="537" t="s">
+      <c r="C10" s="577" t="s">
         <v>394</v>
       </c>
-      <c r="D10" s="549" t="s">
+      <c r="D10" s="578" t="s">
         <v>395</v>
       </c>
       <c r="E10" s="154" t="s">
@@ -17695,10 +17769,10 @@
       <c r="AM10" s="51"/>
     </row>
     <row r="11" spans="1:39" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="553"/>
-      <c r="B11" s="547"/>
-      <c r="C11" s="538"/>
-      <c r="D11" s="550"/>
+      <c r="A11" s="538"/>
+      <c r="B11" s="552"/>
+      <c r="C11" s="554"/>
+      <c r="D11" s="579"/>
       <c r="E11" s="148" t="s">
         <v>390</v>
       </c>
@@ -17785,10 +17859,10 @@
       <c r="AM11" s="51"/>
     </row>
     <row r="12" spans="1:39" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="554"/>
-      <c r="B12" s="548"/>
-      <c r="C12" s="539"/>
-      <c r="D12" s="551"/>
+      <c r="A12" s="550"/>
+      <c r="B12" s="553"/>
+      <c r="C12" s="555"/>
+      <c r="D12" s="580"/>
       <c r="E12" s="151" t="s">
         <v>391</v>
       </c>
@@ -17875,18 +17949,18 @@
       <c r="AM12" s="51"/>
     </row>
     <row r="13" spans="1:39" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="552" t="str">
+      <c r="A13" s="549" t="str">
         <f t="shared" ref="A13:B13" si="0">A7</f>
         <v>All Zones</v>
       </c>
-      <c r="B13" s="546" t="str">
+      <c r="B13" s="551" t="str">
         <f t="shared" si="0"/>
         <v>Retail</v>
       </c>
-      <c r="C13" s="537" t="s">
+      <c r="C13" s="577" t="s">
         <v>396</v>
       </c>
-      <c r="D13" s="543" t="s">
+      <c r="D13" s="556" t="s">
         <v>393</v>
       </c>
       <c r="E13" s="160" t="s">
@@ -17966,10 +18040,10 @@
       </c>
     </row>
     <row r="14" spans="1:39" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="553"/>
-      <c r="B14" s="547"/>
-      <c r="C14" s="538"/>
-      <c r="D14" s="544"/>
+      <c r="A14" s="538"/>
+      <c r="B14" s="552"/>
+      <c r="C14" s="554"/>
+      <c r="D14" s="557"/>
       <c r="E14" s="163" t="s">
         <v>390</v>
       </c>
@@ -18047,10 +18121,10 @@
       </c>
     </row>
     <row r="15" spans="1:39" ht="37.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="554"/>
-      <c r="B15" s="548"/>
-      <c r="C15" s="555"/>
-      <c r="D15" s="545"/>
+      <c r="A15" s="550"/>
+      <c r="B15" s="553"/>
+      <c r="C15" s="581"/>
+      <c r="D15" s="558"/>
       <c r="E15" s="166" t="s">
         <v>391</v>
       </c>
@@ -18128,18 +18202,18 @@
       </c>
     </row>
     <row r="16" spans="1:39" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="552" t="str">
+      <c r="A16" s="549" t="str">
         <f t="shared" ref="A16:B16" si="1">A10</f>
         <v>All Zones</v>
       </c>
-      <c r="B16" s="546" t="str">
+      <c r="B16" s="551" t="str">
         <f t="shared" si="1"/>
         <v>Retail</v>
       </c>
       <c r="C16" s="560" t="s">
         <v>397</v>
       </c>
-      <c r="D16" s="543" t="s">
+      <c r="D16" s="556" t="s">
         <v>393</v>
       </c>
       <c r="E16" s="160" t="s">
@@ -18219,10 +18293,10 @@
       </c>
     </row>
     <row r="17" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="553"/>
-      <c r="B17" s="547"/>
+      <c r="A17" s="538"/>
+      <c r="B17" s="552"/>
       <c r="C17" s="560"/>
-      <c r="D17" s="544"/>
+      <c r="D17" s="557"/>
       <c r="E17" s="163" t="s">
         <v>390</v>
       </c>
@@ -18300,10 +18374,10 @@
       </c>
     </row>
     <row r="18" spans="1:29" ht="37.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="554"/>
-      <c r="B18" s="548"/>
+      <c r="A18" s="550"/>
+      <c r="B18" s="553"/>
       <c r="C18" s="560"/>
-      <c r="D18" s="545"/>
+      <c r="D18" s="558"/>
       <c r="E18" s="166" t="s">
         <v>391</v>
       </c>
@@ -18381,18 +18455,18 @@
       </c>
     </row>
     <row r="19" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="552" t="str">
+      <c r="A19" s="549" t="str">
         <f t="shared" ref="A19:B19" si="2">A13</f>
         <v>All Zones</v>
       </c>
-      <c r="B19" s="546" t="str">
+      <c r="B19" s="551" t="str">
         <f t="shared" si="2"/>
         <v>Retail</v>
       </c>
       <c r="C19" s="561" t="s">
         <v>196</v>
       </c>
-      <c r="D19" s="543" t="s">
+      <c r="D19" s="556" t="s">
         <v>393</v>
       </c>
       <c r="E19" s="160" t="s">
@@ -18472,10 +18546,10 @@
       </c>
     </row>
     <row r="20" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="553"/>
-      <c r="B20" s="547"/>
+      <c r="A20" s="538"/>
+      <c r="B20" s="552"/>
       <c r="C20" s="560"/>
-      <c r="D20" s="544"/>
+      <c r="D20" s="557"/>
       <c r="E20" s="163" t="s">
         <v>390</v>
       </c>
@@ -18553,10 +18627,10 @@
       </c>
     </row>
     <row r="21" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="554"/>
-      <c r="B21" s="548"/>
+      <c r="A21" s="550"/>
+      <c r="B21" s="553"/>
       <c r="C21" s="562"/>
-      <c r="D21" s="545"/>
+      <c r="D21" s="558"/>
       <c r="E21" s="172" t="s">
         <v>391</v>
       </c>
@@ -18634,18 +18708,18 @@
       </c>
     </row>
     <row r="22" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="523" t="str">
+      <c r="A22" s="566" t="str">
         <f t="shared" ref="A22:B22" si="3">A16</f>
         <v>All Zones</v>
       </c>
-      <c r="B22" s="526" t="str">
+      <c r="B22" s="569" t="str">
         <f t="shared" si="3"/>
         <v>Retail</v>
       </c>
-      <c r="C22" s="529" t="s">
+      <c r="C22" s="572" t="s">
         <v>398</v>
       </c>
-      <c r="D22" s="532" t="s">
+      <c r="D22" s="575" t="s">
         <v>393</v>
       </c>
       <c r="E22" s="196" t="s">
@@ -18725,10 +18799,10 @@
       </c>
     </row>
     <row r="23" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="524"/>
-      <c r="B23" s="527"/>
-      <c r="C23" s="530"/>
-      <c r="D23" s="533"/>
+      <c r="A23" s="567"/>
+      <c r="B23" s="570"/>
+      <c r="C23" s="573"/>
+      <c r="D23" s="535"/>
       <c r="E23" s="197" t="s">
         <v>390</v>
       </c>
@@ -18806,10 +18880,10 @@
       </c>
     </row>
     <row r="24" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="525"/>
-      <c r="B24" s="528"/>
-      <c r="C24" s="531"/>
-      <c r="D24" s="534"/>
+      <c r="A24" s="568"/>
+      <c r="B24" s="571"/>
+      <c r="C24" s="574"/>
+      <c r="D24" s="576"/>
       <c r="E24" s="198" t="s">
         <v>391</v>
       </c>
@@ -18887,18 +18961,18 @@
       </c>
     </row>
     <row r="25" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="552" t="str">
+      <c r="A25" s="549" t="str">
         <f t="shared" ref="A25:B25" si="4">A16</f>
         <v>All Zones</v>
       </c>
-      <c r="B25" s="546" t="str">
+      <c r="B25" s="551" t="str">
         <f t="shared" si="4"/>
         <v>Retail</v>
       </c>
-      <c r="C25" s="568" t="s">
+      <c r="C25" s="542" t="s">
         <v>399</v>
       </c>
-      <c r="D25" s="543" t="s">
+      <c r="D25" s="556" t="s">
         <v>393</v>
       </c>
       <c r="E25" s="192" t="s">
@@ -19002,10 +19076,10 @@
       </c>
     </row>
     <row r="26" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="553"/>
-      <c r="B26" s="547"/>
-      <c r="C26" s="538"/>
-      <c r="D26" s="544"/>
+      <c r="A26" s="538"/>
+      <c r="B26" s="552"/>
+      <c r="C26" s="554"/>
+      <c r="D26" s="557"/>
       <c r="E26" s="163" t="s">
         <v>390</v>
       </c>
@@ -19107,10 +19181,10 @@
       </c>
     </row>
     <row r="27" spans="1:29" ht="37.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="554"/>
-      <c r="B27" s="548"/>
-      <c r="C27" s="539"/>
-      <c r="D27" s="545"/>
+      <c r="A27" s="550"/>
+      <c r="B27" s="553"/>
+      <c r="C27" s="555"/>
+      <c r="D27" s="558"/>
       <c r="E27" s="172" t="s">
         <v>391</v>
       </c>
@@ -19212,18 +19286,18 @@
       </c>
     </row>
     <row r="28" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="552" t="str">
+      <c r="A28" s="549" t="str">
         <f t="shared" ref="A28:B28" si="5">A19</f>
         <v>All Zones</v>
       </c>
-      <c r="B28" s="546" t="str">
+      <c r="B28" s="551" t="str">
         <f t="shared" si="5"/>
         <v>Retail</v>
       </c>
-      <c r="C28" s="569" t="s">
+      <c r="C28" s="523" t="s">
         <v>400</v>
       </c>
-      <c r="D28" s="571" t="s">
+      <c r="D28" s="526" t="s">
         <v>393</v>
       </c>
       <c r="E28" s="173" t="s">
@@ -19327,10 +19401,10 @@
       </c>
     </row>
     <row r="29" spans="1:29" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="553"/>
-      <c r="B29" s="547"/>
-      <c r="C29" s="538"/>
-      <c r="D29" s="572"/>
+      <c r="A29" s="538"/>
+      <c r="B29" s="552"/>
+      <c r="C29" s="554"/>
+      <c r="D29" s="527"/>
       <c r="E29" s="176" t="s">
         <v>390</v>
       </c>
@@ -19432,10 +19506,10 @@
       </c>
     </row>
     <row r="30" spans="1:29" ht="37.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="554"/>
-      <c r="B30" s="548"/>
-      <c r="C30" s="570"/>
-      <c r="D30" s="573"/>
+      <c r="A30" s="550"/>
+      <c r="B30" s="553"/>
+      <c r="C30" s="559"/>
+      <c r="D30" s="528"/>
       <c r="E30" s="179" t="s">
         <v>391</v>
       </c>
@@ -19537,47 +19611,47 @@
       </c>
     </row>
     <row r="31" spans="1:29" ht="25.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="563" t="s">
+      <c r="A31" s="543" t="s">
         <v>401</v>
       </c>
-      <c r="B31" s="564"/>
-      <c r="C31" s="564"/>
-      <c r="D31" s="564"/>
-      <c r="E31" s="564"/>
-      <c r="F31" s="564"/>
-      <c r="G31" s="564"/>
-      <c r="H31" s="564"/>
-      <c r="I31" s="564"/>
-      <c r="J31" s="564"/>
-      <c r="K31" s="564"/>
-      <c r="L31" s="564"/>
-      <c r="M31" s="564"/>
-      <c r="N31" s="564"/>
-      <c r="O31" s="564"/>
-      <c r="P31" s="564"/>
-      <c r="Q31" s="564"/>
-      <c r="R31" s="564"/>
-      <c r="S31" s="564"/>
-      <c r="T31" s="564"/>
-      <c r="U31" s="564"/>
-      <c r="V31" s="564"/>
-      <c r="W31" s="564"/>
-      <c r="X31" s="564"/>
-      <c r="Y31" s="564"/>
-      <c r="Z31" s="564"/>
-      <c r="AA31" s="564"/>
-      <c r="AB31" s="564"/>
-      <c r="AC31" s="565"/>
+      <c r="B31" s="544"/>
+      <c r="C31" s="544"/>
+      <c r="D31" s="544"/>
+      <c r="E31" s="544"/>
+      <c r="F31" s="544"/>
+      <c r="G31" s="544"/>
+      <c r="H31" s="544"/>
+      <c r="I31" s="544"/>
+      <c r="J31" s="544"/>
+      <c r="K31" s="544"/>
+      <c r="L31" s="544"/>
+      <c r="M31" s="544"/>
+      <c r="N31" s="544"/>
+      <c r="O31" s="544"/>
+      <c r="P31" s="544"/>
+      <c r="Q31" s="544"/>
+      <c r="R31" s="544"/>
+      <c r="S31" s="544"/>
+      <c r="T31" s="544"/>
+      <c r="U31" s="544"/>
+      <c r="V31" s="544"/>
+      <c r="W31" s="544"/>
+      <c r="X31" s="544"/>
+      <c r="Y31" s="544"/>
+      <c r="Z31" s="544"/>
+      <c r="AA31" s="544"/>
+      <c r="AB31" s="544"/>
+      <c r="AC31" s="545"/>
     </row>
     <row r="32" spans="1:29" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="574"/>
-      <c r="B32" s="581" t="s">
+      <c r="A32" s="520"/>
+      <c r="B32" s="531" t="s">
         <v>99</v>
       </c>
-      <c r="C32" s="569" t="s">
+      <c r="C32" s="523" t="s">
         <v>402</v>
       </c>
-      <c r="D32" s="583"/>
+      <c r="D32" s="534"/>
       <c r="E32" s="183" t="s">
         <v>389</v>
       </c>
@@ -19655,10 +19729,10 @@
       </c>
     </row>
     <row r="33" spans="1:29" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="579"/>
-      <c r="B33" s="541"/>
-      <c r="C33" s="577"/>
-      <c r="D33" s="533"/>
+      <c r="A33" s="529"/>
+      <c r="B33" s="532"/>
+      <c r="C33" s="524"/>
+      <c r="D33" s="535"/>
       <c r="E33" s="182" t="s">
         <v>390</v>
       </c>
@@ -19736,10 +19810,10 @@
       </c>
     </row>
     <row r="34" spans="1:29" ht="28.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="580"/>
-      <c r="B34" s="582"/>
-      <c r="C34" s="578"/>
-      <c r="D34" s="584"/>
+      <c r="A34" s="530"/>
+      <c r="B34" s="533"/>
+      <c r="C34" s="525"/>
+      <c r="D34" s="536"/>
       <c r="E34" s="187" t="s">
         <v>391</v>
       </c>
@@ -19817,14 +19891,14 @@
       </c>
     </row>
     <row r="35" spans="1:29" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="585"/>
-      <c r="B35" s="586" t="s">
+      <c r="A35" s="537"/>
+      <c r="B35" s="540" t="s">
         <v>99</v>
       </c>
-      <c r="C35" s="568" t="s">
+      <c r="C35" s="542" t="s">
         <v>403</v>
       </c>
-      <c r="D35" s="533"/>
+      <c r="D35" s="535"/>
       <c r="E35" s="222" t="s">
         <v>389</v>
       </c>
@@ -19902,10 +19976,10 @@
       </c>
     </row>
     <row r="36" spans="1:29" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="553"/>
-      <c r="B36" s="541"/>
-      <c r="C36" s="577"/>
-      <c r="D36" s="533"/>
+      <c r="A36" s="538"/>
+      <c r="B36" s="532"/>
+      <c r="C36" s="524"/>
+      <c r="D36" s="535"/>
       <c r="E36" s="182" t="s">
         <v>390</v>
       </c>
@@ -19983,10 +20057,10 @@
       </c>
     </row>
     <row r="37" spans="1:29" ht="28.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="567"/>
-      <c r="B37" s="542"/>
-      <c r="C37" s="577"/>
-      <c r="D37" s="533"/>
+      <c r="A37" s="539"/>
+      <c r="B37" s="541"/>
+      <c r="C37" s="524"/>
+      <c r="D37" s="535"/>
       <c r="E37" s="223" t="s">
         <v>391</v>
       </c>
@@ -20064,16 +20138,16 @@
       </c>
     </row>
     <row r="38" spans="1:29" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="574" t="s">
+      <c r="A38" s="520" t="s">
         <v>404</v>
       </c>
-      <c r="B38" s="569" t="s">
+      <c r="B38" s="523" t="s">
         <v>99</v>
       </c>
-      <c r="C38" s="569" t="s">
+      <c r="C38" s="523" t="s">
         <v>405</v>
       </c>
-      <c r="D38" s="571" t="s">
+      <c r="D38" s="526" t="s">
         <v>406</v>
       </c>
       <c r="E38" s="183" t="s">
@@ -20153,10 +20227,10 @@
       </c>
     </row>
     <row r="39" spans="1:29" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="575"/>
-      <c r="B39" s="577"/>
-      <c r="C39" s="577"/>
-      <c r="D39" s="572"/>
+      <c r="A39" s="521"/>
+      <c r="B39" s="524"/>
+      <c r="C39" s="524"/>
+      <c r="D39" s="527"/>
       <c r="E39" s="182" t="s">
         <v>390</v>
       </c>
@@ -20234,10 +20308,10 @@
       </c>
     </row>
     <row r="40" spans="1:29" ht="28.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="576"/>
-      <c r="B40" s="578"/>
-      <c r="C40" s="578"/>
-      <c r="D40" s="573"/>
+      <c r="A40" s="522"/>
+      <c r="B40" s="525"/>
+      <c r="C40" s="525"/>
+      <c r="D40" s="528"/>
       <c r="E40" s="187" t="s">
         <v>391</v>
       </c>
@@ -20459,18 +20533,34 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="A38:A40"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="D38:D40"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="D32:D34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="C35:C37"/>
-    <mergeCell ref="D35:D37"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="F2:AC2"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="D19:D21"/>
     <mergeCell ref="A31:AC31"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="A1:AC1"/>
@@ -20487,34 +20577,18 @@
     <mergeCell ref="D28:D30"/>
     <mergeCell ref="A16:A18"/>
     <mergeCell ref="B16:B18"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="D19:D21"/>
-    <mergeCell ref="F2:AC2"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="D22:D24"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="D38:D40"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="D32:D34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="D35:D37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -20550,34 +20624,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="591" t="str">
+      <c r="A1" s="588" t="str">
         <f>"CalBEM Energy Consumption - "&amp;Prototype!A2</f>
         <v>CalBEM Energy Consumption - RetailStripMall</v>
       </c>
-      <c r="B1" s="478"/>
-      <c r="C1" s="478"/>
-      <c r="D1" s="478"/>
-      <c r="E1" s="478"/>
-      <c r="F1" s="478"/>
-      <c r="G1" s="478"/>
-      <c r="H1" s="478"/>
-      <c r="I1" s="592" t="s">
+      <c r="B1" s="479"/>
+      <c r="C1" s="479"/>
+      <c r="D1" s="479"/>
+      <c r="E1" s="479"/>
+      <c r="F1" s="479"/>
+      <c r="G1" s="479"/>
+      <c r="H1" s="479"/>
+      <c r="I1" s="589" t="s">
         <v>408</v>
       </c>
-      <c r="J1" s="592"/>
-      <c r="K1" s="592"/>
-      <c r="L1" s="592"/>
-      <c r="N1" s="590" t="s">
+      <c r="J1" s="589"/>
+      <c r="K1" s="589"/>
+      <c r="L1" s="589"/>
+      <c r="N1" s="587" t="s">
         <v>409</v>
       </c>
-      <c r="O1" s="441"/>
-      <c r="P1" s="441"/>
-      <c r="Q1" s="441"/>
-      <c r="R1" s="441"/>
-      <c r="S1" s="441"/>
-      <c r="T1" s="441"/>
-      <c r="U1" s="441"/>
-      <c r="V1" s="441"/>
+      <c r="O1" s="442"/>
+      <c r="P1" s="442"/>
+      <c r="Q1" s="442"/>
+      <c r="R1" s="442"/>
+      <c r="S1" s="442"/>
+      <c r="T1" s="442"/>
+      <c r="U1" s="442"/>
+      <c r="V1" s="442"/>
       <c r="Y1" s="3" t="s">
         <v>410</v>
       </c>
@@ -20654,7 +20728,7 @@
       </c>
     </row>
     <row r="3" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="588" t="s">
+      <c r="A3" s="585" t="s">
         <v>55</v>
       </c>
       <c r="B3" s="420">
@@ -20681,7 +20755,7 @@
         <f>J3-K3</f>
         <v>23.400000000000006</v>
       </c>
-      <c r="N3" s="587" t="s">
+      <c r="N3" s="584" t="s">
         <v>117</v>
       </c>
       <c r="O3" s="200">
@@ -20714,7 +20788,7 @@
       </c>
     </row>
     <row r="4" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="588"/>
+      <c r="A4" s="585"/>
       <c r="B4" s="420">
         <v>2</v>
       </c>
@@ -20739,7 +20813,7 @@
         <f t="shared" ref="L4:L18" si="2">J4-K4</f>
         <v>29.200000000000003</v>
       </c>
-      <c r="N4" s="587"/>
+      <c r="N4" s="584"/>
       <c r="O4" s="200">
         <v>2</v>
       </c>
@@ -20770,7 +20844,7 @@
       </c>
     </row>
     <row r="5" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="588"/>
+      <c r="A5" s="585"/>
       <c r="B5" s="420">
         <v>3</v>
       </c>
@@ -20795,7 +20869,7 @@
         <f t="shared" si="2"/>
         <v>26.150000000000006</v>
       </c>
-      <c r="N5" s="587"/>
+      <c r="N5" s="584"/>
       <c r="O5" s="200">
         <v>3</v>
       </c>
@@ -20826,7 +20900,7 @@
       </c>
     </row>
     <row r="6" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="588"/>
+      <c r="A6" s="585"/>
       <c r="B6" s="420">
         <v>4</v>
       </c>
@@ -20851,7 +20925,7 @@
         <f t="shared" si="2"/>
         <v>30.450000000000003</v>
       </c>
-      <c r="N6" s="587"/>
+      <c r="N6" s="584"/>
       <c r="O6" s="200">
         <v>4</v>
       </c>
@@ -20882,7 +20956,7 @@
       </c>
     </row>
     <row r="7" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="588"/>
+      <c r="A7" s="585"/>
       <c r="B7" s="420">
         <v>5</v>
       </c>
@@ -20907,7 +20981,7 @@
         <f t="shared" si="2"/>
         <v>25.200000000000003</v>
       </c>
-      <c r="N7" s="587"/>
+      <c r="N7" s="584"/>
       <c r="O7" s="200">
         <v>5</v>
       </c>
@@ -20938,7 +21012,7 @@
       </c>
     </row>
     <row r="8" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="588"/>
+      <c r="A8" s="585"/>
       <c r="B8" s="420">
         <v>6</v>
       </c>
@@ -20963,7 +21037,7 @@
         <f t="shared" si="2"/>
         <v>28.900000000000006</v>
       </c>
-      <c r="N8" s="587"/>
+      <c r="N8" s="584"/>
       <c r="O8" s="200">
         <v>6</v>
       </c>
@@ -20994,7 +21068,7 @@
       </c>
     </row>
     <row r="9" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="588"/>
+      <c r="A9" s="585"/>
       <c r="B9" s="420">
         <v>7</v>
       </c>
@@ -21019,7 +21093,7 @@
         <f t="shared" si="2"/>
         <v>28.900000000000006</v>
       </c>
-      <c r="N9" s="587"/>
+      <c r="N9" s="584"/>
       <c r="O9" s="200">
         <v>7</v>
       </c>
@@ -21050,7 +21124,7 @@
       </c>
     </row>
     <row r="10" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="588"/>
+      <c r="A10" s="585"/>
       <c r="B10" s="420">
         <v>8</v>
       </c>
@@ -21075,7 +21149,7 @@
         <f t="shared" si="2"/>
         <v>29.450000000000003</v>
       </c>
-      <c r="N10" s="587"/>
+      <c r="N10" s="584"/>
       <c r="O10" s="200">
         <v>8</v>
       </c>
@@ -21106,7 +21180,7 @@
       </c>
     </row>
     <row r="11" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="588"/>
+      <c r="A11" s="585"/>
       <c r="B11" s="420">
         <v>9</v>
       </c>
@@ -21131,7 +21205,7 @@
         <f t="shared" si="2"/>
         <v>29.799999999999997</v>
       </c>
-      <c r="N11" s="587"/>
+      <c r="N11" s="584"/>
       <c r="O11" s="200">
         <v>9</v>
       </c>
@@ -21162,7 +21236,7 @@
       </c>
     </row>
     <row r="12" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="588"/>
+      <c r="A12" s="585"/>
       <c r="B12" s="420">
         <v>10</v>
       </c>
@@ -21187,7 +21261,7 @@
         <f t="shared" si="2"/>
         <v>30.099999999999994</v>
       </c>
-      <c r="N12" s="587"/>
+      <c r="N12" s="584"/>
       <c r="O12" s="200">
         <v>10</v>
       </c>
@@ -21218,7 +21292,7 @@
       </c>
     </row>
     <row r="13" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="588"/>
+      <c r="A13" s="585"/>
       <c r="B13" s="420">
         <v>11</v>
       </c>
@@ -21243,7 +21317,7 @@
         <f t="shared" si="2"/>
         <v>31.150000000000006</v>
       </c>
-      <c r="N13" s="587"/>
+      <c r="N13" s="584"/>
       <c r="O13" s="200">
         <v>11</v>
       </c>
@@ -21274,7 +21348,7 @@
       </c>
     </row>
     <row r="14" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="588"/>
+      <c r="A14" s="585"/>
       <c r="B14" s="420">
         <v>12</v>
       </c>
@@ -21299,7 +21373,7 @@
         <f t="shared" si="2"/>
         <v>30.650000000000006</v>
       </c>
-      <c r="N14" s="587"/>
+      <c r="N14" s="584"/>
       <c r="O14" s="200">
         <v>12</v>
       </c>
@@ -21330,7 +21404,7 @@
       </c>
     </row>
     <row r="15" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="588"/>
+      <c r="A15" s="585"/>
       <c r="B15" s="420">
         <v>13</v>
       </c>
@@ -21355,7 +21429,7 @@
         <f t="shared" si="2"/>
         <v>31.150000000000006</v>
       </c>
-      <c r="N15" s="587"/>
+      <c r="N15" s="584"/>
       <c r="O15" s="200">
         <v>13</v>
       </c>
@@ -21386,7 +21460,7 @@
       </c>
     </row>
     <row r="16" spans="1:35" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="588"/>
+      <c r="A16" s="585"/>
       <c r="B16" s="420">
         <v>14</v>
       </c>
@@ -21411,7 +21485,7 @@
         <f t="shared" si="2"/>
         <v>31.299999999999997</v>
       </c>
-      <c r="N16" s="587"/>
+      <c r="N16" s="584"/>
       <c r="O16" s="200">
         <v>14</v>
       </c>
@@ -21442,7 +21516,7 @@
       </c>
     </row>
     <row r="17" spans="1:22" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="588"/>
+      <c r="A17" s="585"/>
       <c r="B17" s="420">
         <v>15</v>
       </c>
@@ -21467,7 +21541,7 @@
         <f t="shared" si="2"/>
         <v>30.049999999999997</v>
       </c>
-      <c r="N17" s="587"/>
+      <c r="N17" s="584"/>
       <c r="O17" s="200">
         <v>15</v>
       </c>
@@ -21498,7 +21572,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="589"/>
+      <c r="A18" s="586"/>
       <c r="B18" s="431">
         <v>16</v>
       </c>
@@ -21523,7 +21597,7 @@
         <f t="shared" si="2"/>
         <v>30.599999999999994</v>
       </c>
-      <c r="N18" s="587"/>
+      <c r="N18" s="584"/>
       <c r="O18" s="200">
         <v>16</v>
       </c>
@@ -21609,80 +21683,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="28.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="459" t="str">
+      <c r="A1" s="463" t="str">
         <f>"% of Floor Area per CZ and Vintage Bin - Retail"</f>
         <v>% of Floor Area per CZ and Vintage Bin - Retail</v>
       </c>
-      <c r="B1" s="459"/>
-      <c r="C1" s="459"/>
-      <c r="D1" s="459"/>
-      <c r="E1" s="459"/>
-      <c r="F1" s="459"/>
-      <c r="G1" s="459"/>
-      <c r="J1" s="459" t="str">
+      <c r="B1" s="463"/>
+      <c r="C1" s="463"/>
+      <c r="D1" s="463"/>
+      <c r="E1" s="463"/>
+      <c r="F1" s="463"/>
+      <c r="G1" s="463"/>
+      <c r="J1" s="463" t="str">
         <f>"% of Floor Area per CZ and Vintage Bin - Retail"</f>
         <v>% of Floor Area per CZ and Vintage Bin - Retail</v>
       </c>
-      <c r="K1" s="459"/>
-      <c r="L1" s="459"/>
-      <c r="M1" s="459"/>
-      <c r="N1" s="459"/>
-      <c r="O1" s="459"/>
-      <c r="P1" s="459"/>
-      <c r="Q1" s="459"/>
-      <c r="R1" s="459"/>
-      <c r="S1" s="459"/>
-      <c r="T1" s="459"/>
-      <c r="U1" s="459"/>
-      <c r="V1" s="459"/>
-      <c r="W1" s="459"/>
-      <c r="X1" s="459"/>
-      <c r="Y1" s="459"/>
-      <c r="Z1" s="459"/>
-      <c r="AA1" s="459"/>
+      <c r="K1" s="463"/>
+      <c r="L1" s="463"/>
+      <c r="M1" s="463"/>
+      <c r="N1" s="463"/>
+      <c r="O1" s="463"/>
+      <c r="P1" s="463"/>
+      <c r="Q1" s="463"/>
+      <c r="R1" s="463"/>
+      <c r="S1" s="463"/>
+      <c r="T1" s="463"/>
+      <c r="U1" s="463"/>
+      <c r="V1" s="463"/>
+      <c r="W1" s="463"/>
+      <c r="X1" s="463"/>
+      <c r="Y1" s="463"/>
+      <c r="Z1" s="463"/>
+      <c r="AA1" s="463"/>
     </row>
     <row r="2" spans="1:28" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="599" t="s">
+      <c r="A2" s="596" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="599" t="s">
+      <c r="B2" s="596" t="s">
         <v>412</v>
       </c>
-      <c r="C2" s="599" t="s">
+      <c r="C2" s="596" t="s">
         <v>432</v>
       </c>
-      <c r="D2" s="599"/>
-      <c r="E2" s="599"/>
-      <c r="F2" s="599"/>
-      <c r="G2" s="599"/>
-      <c r="J2" s="599" t="s">
+      <c r="D2" s="596"/>
+      <c r="E2" s="596"/>
+      <c r="F2" s="596"/>
+      <c r="G2" s="596"/>
+      <c r="J2" s="596" t="s">
         <v>143</v>
       </c>
-      <c r="K2" s="599" t="s">
+      <c r="K2" s="596" t="s">
         <v>432</v>
       </c>
-      <c r="L2" s="599" t="s">
+      <c r="L2" s="596" t="s">
         <v>412</v>
       </c>
-      <c r="M2" s="599"/>
-      <c r="N2" s="599"/>
-      <c r="O2" s="599"/>
-      <c r="P2" s="599"/>
-      <c r="Q2" s="599"/>
-      <c r="R2" s="599"/>
-      <c r="S2" s="599"/>
-      <c r="T2" s="599"/>
-      <c r="U2" s="599"/>
-      <c r="V2" s="599"/>
-      <c r="W2" s="599"/>
-      <c r="X2" s="599"/>
-      <c r="Y2" s="599"/>
-      <c r="Z2" s="599"/>
-      <c r="AA2" s="599"/>
+      <c r="M2" s="596"/>
+      <c r="N2" s="596"/>
+      <c r="O2" s="596"/>
+      <c r="P2" s="596"/>
+      <c r="Q2" s="596"/>
+      <c r="R2" s="596"/>
+      <c r="S2" s="596"/>
+      <c r="T2" s="596"/>
+      <c r="U2" s="596"/>
+      <c r="V2" s="596"/>
+      <c r="W2" s="596"/>
+      <c r="X2" s="596"/>
+      <c r="Y2" s="596"/>
+      <c r="Z2" s="596"/>
+      <c r="AA2" s="596"/>
     </row>
     <row r="3" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="599"/>
-      <c r="B3" s="599"/>
+      <c r="A3" s="596"/>
+      <c r="B3" s="596"/>
       <c r="C3" s="347" t="s">
         <v>433</v>
       </c>
@@ -21696,8 +21770,8 @@
         <v>177</v>
       </c>
       <c r="G3" s="347"/>
-      <c r="J3" s="599"/>
-      <c r="K3" s="599"/>
+      <c r="J3" s="596"/>
+      <c r="K3" s="596"/>
       <c r="L3" s="327">
         <v>1</v>
       </c>
@@ -21748,7 +21822,7 @@
       </c>
     </row>
     <row r="4" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="596" t="s">
+      <c r="A4" s="593" t="s">
         <v>117</v>
       </c>
       <c r="B4" s="344">
@@ -21763,7 +21837,7 @@
         <f>SUM(C4:F4)</f>
         <v>0</v>
       </c>
-      <c r="J4" s="593" t="s">
+      <c r="J4" s="590" t="s">
         <v>117</v>
       </c>
       <c r="K4" s="36" t="s">
@@ -21791,7 +21865,7 @@
       </c>
     </row>
     <row r="5" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="597"/>
+      <c r="A5" s="594"/>
       <c r="B5" s="345">
         <v>2</v>
       </c>
@@ -21804,7 +21878,7 @@
         <f t="shared" ref="H5:H20" si="1">SUM(C5:F5)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="594"/>
+      <c r="J5" s="591"/>
       <c r="K5" s="36" t="s">
         <v>173</v>
       </c>
@@ -21830,7 +21904,7 @@
       </c>
     </row>
     <row r="6" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="597"/>
+      <c r="A6" s="594"/>
       <c r="B6" s="345">
         <v>3</v>
       </c>
@@ -21843,7 +21917,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J6" s="594"/>
+      <c r="J6" s="591"/>
       <c r="K6" s="36" t="s">
         <v>175</v>
       </c>
@@ -21869,7 +21943,7 @@
       </c>
     </row>
     <row r="7" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="597"/>
+      <c r="A7" s="594"/>
       <c r="B7" s="345">
         <v>4</v>
       </c>
@@ -21882,7 +21956,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J7" s="594"/>
+      <c r="J7" s="591"/>
       <c r="K7" s="36" t="s">
         <v>177</v>
       </c>
@@ -21908,7 +21982,7 @@
       </c>
     </row>
     <row r="8" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="597"/>
+      <c r="A8" s="594"/>
       <c r="B8" s="345">
         <v>5</v>
       </c>
@@ -21921,7 +21995,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J8" s="594"/>
+      <c r="J8" s="591"/>
       <c r="K8" s="36" t="s">
         <v>434</v>
       </c>
@@ -21947,7 +22021,7 @@
       </c>
     </row>
     <row r="9" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="597"/>
+      <c r="A9" s="594"/>
       <c r="B9" s="345">
         <v>6</v>
       </c>
@@ -21960,7 +22034,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J9" s="595"/>
+      <c r="J9" s="592"/>
       <c r="K9" s="36" t="s">
         <v>293</v>
       </c>
@@ -21986,7 +22060,7 @@
       </c>
     </row>
     <row r="10" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="597"/>
+      <c r="A10" s="594"/>
       <c r="B10" s="345">
         <v>7</v>
       </c>
@@ -22008,7 +22082,7 @@
       <c r="P10" s="59"/>
     </row>
     <row r="11" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="597"/>
+      <c r="A11" s="594"/>
       <c r="B11" s="345">
         <v>8</v>
       </c>
@@ -22030,7 +22104,7 @@
       <c r="P11" s="59"/>
     </row>
     <row r="12" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="597"/>
+      <c r="A12" s="594"/>
       <c r="B12" s="345">
         <v>9</v>
       </c>
@@ -22052,7 +22126,7 @@
       <c r="P12" s="59"/>
     </row>
     <row r="13" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="597"/>
+      <c r="A13" s="594"/>
       <c r="B13" s="345">
         <v>10</v>
       </c>
@@ -22074,7 +22148,7 @@
       <c r="P13" s="59"/>
     </row>
     <row r="14" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="597"/>
+      <c r="A14" s="594"/>
       <c r="B14" s="345">
         <v>11</v>
       </c>
@@ -22096,7 +22170,7 @@
       <c r="P14" s="59"/>
     </row>
     <row r="15" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="597"/>
+      <c r="A15" s="594"/>
       <c r="B15" s="345">
         <v>12</v>
       </c>
@@ -22118,7 +22192,7 @@
       <c r="P15" s="59"/>
     </row>
     <row r="16" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="597"/>
+      <c r="A16" s="594"/>
       <c r="B16" s="345">
         <v>13</v>
       </c>
@@ -22140,7 +22214,7 @@
       <c r="P16" s="59"/>
     </row>
     <row r="17" spans="1:16" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="597"/>
+      <c r="A17" s="594"/>
       <c r="B17" s="345">
         <v>14</v>
       </c>
@@ -22162,7 +22236,7 @@
       <c r="P17" s="59"/>
     </row>
     <row r="18" spans="1:16" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="597"/>
+      <c r="A18" s="594"/>
       <c r="B18" s="345">
         <v>15</v>
       </c>
@@ -22184,7 +22258,7 @@
       <c r="P18" s="59"/>
     </row>
     <row r="19" spans="1:16" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="597"/>
+      <c r="A19" s="594"/>
       <c r="B19" s="345">
         <v>16</v>
       </c>
@@ -22206,7 +22280,7 @@
       <c r="P19" s="59"/>
     </row>
     <row r="20" spans="1:16" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="598"/>
+      <c r="A20" s="595"/>
       <c r="B20" s="346" t="s">
         <v>435</v>
       </c>
@@ -22320,19 +22394,19 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="459" t="str">
+      <c r="A1" s="463" t="str">
         <f>"PV - "&amp;Prototype!A2</f>
         <v>PV - RetailStripMall</v>
       </c>
-      <c r="B1" s="459"/>
-      <c r="C1" s="459"/>
-      <c r="D1" s="459"/>
-      <c r="E1" s="459"/>
-      <c r="F1" s="459"/>
-      <c r="G1" s="459"/>
-      <c r="H1" s="459"/>
-      <c r="I1" s="459"/>
-      <c r="J1" s="459"/>
+      <c r="B1" s="463"/>
+      <c r="C1" s="463"/>
+      <c r="D1" s="463"/>
+      <c r="E1" s="463"/>
+      <c r="F1" s="463"/>
+      <c r="G1" s="463"/>
+      <c r="H1" s="463"/>
+      <c r="I1" s="463"/>
+      <c r="J1" s="463"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -22386,17 +22460,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="459" t="str">
+      <c r="A1" s="463" t="str">
         <f>"EV Charger - "&amp;Prototype!A2</f>
         <v>EV Charger - RetailStripMall</v>
       </c>
-      <c r="B1" s="459"/>
-      <c r="C1" s="459"/>
-      <c r="D1" s="459"/>
-      <c r="E1" s="459"/>
-      <c r="F1" s="459"/>
-      <c r="G1" s="459"/>
-      <c r="H1" s="459"/>
+      <c r="B1" s="463"/>
+      <c r="C1" s="463"/>
+      <c r="D1" s="463"/>
+      <c r="E1" s="463"/>
+      <c r="F1" s="463"/>
+      <c r="G1" s="463"/>
+      <c r="H1" s="463"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -22450,12 +22524,12 @@
       <c r="C1" t="s">
         <v>439</v>
       </c>
-      <c r="D1" s="600" t="s">
+      <c r="D1" s="597" t="s">
         <v>440</v>
       </c>
-      <c r="E1" s="600"/>
-      <c r="F1" s="600"/>
-      <c r="G1" s="600"/>
+      <c r="E1" s="597"/>
+      <c r="F1" s="597"/>
+      <c r="G1" s="597"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="319" t="s">
@@ -23318,24 +23392,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="441" t="str">
+      <c r="A1" s="442" t="str">
         <f>"Proposed Layout - "&amp;Prototype!A2</f>
         <v>Proposed Layout - RetailStripMall</v>
       </c>
-      <c r="B1" s="441"/>
-      <c r="C1" s="441"/>
-      <c r="D1" s="441"/>
-      <c r="E1" s="441"/>
-      <c r="F1" s="441"/>
-      <c r="G1" s="441"/>
-      <c r="H1" s="441"/>
-      <c r="I1" s="441"/>
-      <c r="J1" s="441"/>
-      <c r="K1" s="441"/>
-      <c r="L1" s="441"/>
-      <c r="M1" s="441"/>
-      <c r="N1" s="441"/>
-      <c r="O1" s="441"/>
+      <c r="B1" s="442"/>
+      <c r="C1" s="442"/>
+      <c r="D1" s="442"/>
+      <c r="E1" s="442"/>
+      <c r="F1" s="442"/>
+      <c r="G1" s="442"/>
+      <c r="H1" s="442"/>
+      <c r="I1" s="442"/>
+      <c r="J1" s="442"/>
+      <c r="K1" s="442"/>
+      <c r="L1" s="442"/>
+      <c r="M1" s="442"/>
+      <c r="N1" s="442"/>
+      <c r="O1" s="442"/>
     </row>
     <row r="2" spans="1:20" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="355" t="s">
@@ -23929,33 +24003,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="459" t="str">
+      <c r="A1" s="463" t="str">
         <f>"Envelope - "&amp;Prototype!A2</f>
         <v>Envelope - RetailStripMall</v>
       </c>
-      <c r="B1" s="459"/>
-      <c r="C1" s="459"/>
-      <c r="D1" s="459"/>
-      <c r="E1" s="459"/>
-      <c r="F1" s="459"/>
-      <c r="G1" s="459"/>
-      <c r="H1" s="459"/>
-      <c r="I1" s="459"/>
-      <c r="J1" s="459"/>
-      <c r="K1" s="459"/>
-      <c r="L1" s="459"/>
-      <c r="M1" s="459"/>
-      <c r="N1" s="459"/>
-      <c r="O1" s="459"/>
-      <c r="P1" s="459"/>
-      <c r="Q1" s="459"/>
-      <c r="R1" s="459"/>
-      <c r="S1" s="459"/>
-      <c r="T1" s="459"/>
-      <c r="U1" s="459"/>
-      <c r="V1" s="459"/>
-      <c r="W1" s="459"/>
-      <c r="X1" s="459"/>
+      <c r="B1" s="463"/>
+      <c r="C1" s="463"/>
+      <c r="D1" s="463"/>
+      <c r="E1" s="463"/>
+      <c r="F1" s="463"/>
+      <c r="G1" s="463"/>
+      <c r="H1" s="463"/>
+      <c r="I1" s="463"/>
+      <c r="J1" s="463"/>
+      <c r="K1" s="463"/>
+      <c r="L1" s="463"/>
+      <c r="M1" s="463"/>
+      <c r="N1" s="463"/>
+      <c r="O1" s="463"/>
+      <c r="P1" s="463"/>
+      <c r="Q1" s="463"/>
+      <c r="R1" s="463"/>
+      <c r="S1" s="463"/>
+      <c r="T1" s="463"/>
+      <c r="U1" s="463"/>
+      <c r="V1" s="463"/>
+      <c r="W1" s="463"/>
+      <c r="X1" s="463"/>
     </row>
     <row r="2" spans="1:25" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="66" t="s">
@@ -24032,19 +24106,19 @@
       </c>
     </row>
     <row r="3" spans="1:25" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="460" t="s">
+      <c r="A3" s="454" t="s">
         <v>166</v>
       </c>
-      <c r="B3" s="460" t="s">
+      <c r="B3" s="454" t="s">
         <v>167</v>
       </c>
-      <c r="C3" s="458" t="s">
+      <c r="C3" s="455" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="458" t="s">
+      <c r="D3" s="455" t="s">
         <v>169</v>
       </c>
-      <c r="E3" s="460" t="s">
+      <c r="E3" s="454" t="s">
         <v>170</v>
       </c>
       <c r="F3" s="315" t="s">
@@ -24106,11 +24180,11 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="460"/>
-      <c r="B4" s="460"/>
-      <c r="C4" s="458"/>
-      <c r="D4" s="458"/>
-      <c r="E4" s="460"/>
+      <c r="A4" s="454"/>
+      <c r="B4" s="454"/>
+      <c r="C4" s="455"/>
+      <c r="D4" s="455"/>
+      <c r="E4" s="454"/>
       <c r="F4" s="302" t="s">
         <v>173</v>
       </c>
@@ -24171,11 +24245,11 @@
       <c r="Y4" s="88"/>
     </row>
     <row r="5" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="460"/>
-      <c r="B5" s="460"/>
-      <c r="C5" s="458"/>
-      <c r="D5" s="458"/>
-      <c r="E5" s="460"/>
+      <c r="A5" s="454"/>
+      <c r="B5" s="454"/>
+      <c r="C5" s="455"/>
+      <c r="D5" s="455"/>
+      <c r="E5" s="454"/>
       <c r="F5" s="305" t="s">
         <v>175</v>
       </c>
@@ -24236,11 +24310,11 @@
       <c r="Y5" s="73"/>
     </row>
     <row r="6" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="460"/>
-      <c r="B6" s="460"/>
-      <c r="C6" s="458"/>
-      <c r="D6" s="458"/>
-      <c r="E6" s="460"/>
+      <c r="A6" s="454"/>
+      <c r="B6" s="454"/>
+      <c r="C6" s="455"/>
+      <c r="D6" s="455"/>
+      <c r="E6" s="454"/>
       <c r="F6" s="307" t="s">
         <v>177</v>
       </c>
@@ -24301,11 +24375,11 @@
       <c r="Y6" s="73"/>
     </row>
     <row r="7" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="460"/>
-      <c r="B7" s="460"/>
-      <c r="C7" s="458"/>
-      <c r="D7" s="458"/>
-      <c r="E7" s="460"/>
+      <c r="A7" s="454"/>
+      <c r="B7" s="454"/>
+      <c r="C7" s="455"/>
+      <c r="D7" s="455"/>
+      <c r="E7" s="454"/>
       <c r="F7" s="309" t="s">
         <v>180</v>
       </c>
@@ -24366,19 +24440,19 @@
       <c r="Y7" s="73"/>
     </row>
     <row r="8" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="460" t="s">
+      <c r="A8" s="454" t="s">
         <v>181</v>
       </c>
-      <c r="B8" s="460" t="s">
+      <c r="B8" s="454" t="s">
         <v>167</v>
       </c>
-      <c r="C8" s="458" t="s">
+      <c r="C8" s="455" t="s">
         <v>182</v>
       </c>
-      <c r="D8" s="461" t="s">
+      <c r="D8" s="464" t="s">
         <v>183</v>
       </c>
-      <c r="E8" s="460" t="s">
+      <c r="E8" s="454" t="s">
         <v>170</v>
       </c>
       <c r="F8" s="315" t="s">
@@ -24387,7 +24461,7 @@
       <c r="G8" s="315" t="s">
         <v>80</v>
       </c>
-      <c r="H8" s="458" t="s">
+      <c r="H8" s="455" t="s">
         <v>184</v>
       </c>
       <c r="I8" s="312">
@@ -24441,18 +24515,18 @@
       <c r="Y8" s="73"/>
     </row>
     <row r="9" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="460"/>
-      <c r="B9" s="460"/>
-      <c r="C9" s="458"/>
-      <c r="D9" s="461"/>
-      <c r="E9" s="460"/>
+      <c r="A9" s="454"/>
+      <c r="B9" s="454"/>
+      <c r="C9" s="455"/>
+      <c r="D9" s="464"/>
+      <c r="E9" s="454"/>
       <c r="F9" s="302" t="s">
         <v>173</v>
       </c>
       <c r="G9" s="302">
         <v>1992</v>
       </c>
-      <c r="H9" s="458"/>
+      <c r="H9" s="455"/>
       <c r="I9" s="304">
         <v>5.7000000000000002E-2</v>
       </c>
@@ -24504,11 +24578,11 @@
       <c r="Y9" s="73"/>
     </row>
     <row r="10" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="460"/>
-      <c r="B10" s="460"/>
-      <c r="C10" s="458"/>
-      <c r="D10" s="461"/>
-      <c r="E10" s="460"/>
+      <c r="A10" s="454"/>
+      <c r="B10" s="454"/>
+      <c r="C10" s="455"/>
+      <c r="D10" s="464"/>
+      <c r="E10" s="454"/>
       <c r="F10" s="305" t="s">
         <v>175</v>
       </c>
@@ -24569,11 +24643,11 @@
       <c r="Y10" s="73"/>
     </row>
     <row r="11" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="460"/>
-      <c r="B11" s="460"/>
-      <c r="C11" s="458"/>
-      <c r="D11" s="461"/>
-      <c r="E11" s="460"/>
+      <c r="A11" s="454"/>
+      <c r="B11" s="454"/>
+      <c r="C11" s="455"/>
+      <c r="D11" s="464"/>
+      <c r="E11" s="454"/>
       <c r="F11" s="307" t="s">
         <v>177</v>
       </c>
@@ -24634,11 +24708,11 @@
       <c r="Y11" s="73"/>
     </row>
     <row r="12" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="460"/>
-      <c r="B12" s="460"/>
-      <c r="C12" s="458"/>
-      <c r="D12" s="461"/>
-      <c r="E12" s="460"/>
+      <c r="A12" s="454"/>
+      <c r="B12" s="454"/>
+      <c r="C12" s="455"/>
+      <c r="D12" s="464"/>
+      <c r="E12" s="454"/>
       <c r="F12" s="309" t="s">
         <v>180</v>
       </c>
@@ -24699,19 +24773,19 @@
       <c r="Y12" s="73"/>
     </row>
     <row r="13" spans="1:25" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="460" t="s">
+      <c r="A13" s="454" t="s">
         <v>187</v>
       </c>
-      <c r="B13" s="460" t="s">
+      <c r="B13" s="454" t="s">
         <v>167</v>
       </c>
-      <c r="C13" s="458" t="s">
+      <c r="C13" s="455" t="s">
         <v>188</v>
       </c>
-      <c r="D13" s="458" t="s">
+      <c r="D13" s="455" t="s">
         <v>189</v>
       </c>
-      <c r="E13" s="460" t="s">
+      <c r="E13" s="454" t="s">
         <v>170</v>
       </c>
       <c r="F13" s="302" t="s">
@@ -24720,7 +24794,7 @@
       <c r="G13" s="302" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="458" t="s">
+      <c r="H13" s="455" t="s">
         <v>190</v>
       </c>
       <c r="I13" s="315">
@@ -24790,18 +24864,18 @@
       <c r="Y13" s="73"/>
     </row>
     <row r="14" spans="1:25" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="460"/>
-      <c r="B14" s="460"/>
-      <c r="C14" s="458"/>
-      <c r="D14" s="458"/>
-      <c r="E14" s="460"/>
+      <c r="A14" s="454"/>
+      <c r="B14" s="454"/>
+      <c r="C14" s="455"/>
+      <c r="D14" s="455"/>
+      <c r="E14" s="454"/>
       <c r="F14" s="305" t="s">
         <v>173</v>
       </c>
       <c r="G14" s="305" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="458"/>
+      <c r="H14" s="455"/>
       <c r="I14" s="313">
         <f>I13</f>
         <v>0.74</v>
@@ -24869,13 +24943,13 @@
       <c r="Y14" s="73"/>
     </row>
     <row r="15" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="460"/>
-      <c r="B15" s="460"/>
-      <c r="C15" s="458"/>
-      <c r="D15" s="460" t="s">
+      <c r="A15" s="454"/>
+      <c r="B15" s="454"/>
+      <c r="C15" s="455"/>
+      <c r="D15" s="454" t="s">
         <v>191</v>
       </c>
-      <c r="E15" s="460"/>
+      <c r="E15" s="454"/>
       <c r="F15" s="307" t="s">
         <v>175</v>
       </c>
@@ -24936,11 +25010,11 @@
       <c r="Y15" s="73"/>
     </row>
     <row r="16" spans="1:25" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="460"/>
-      <c r="B16" s="460"/>
-      <c r="C16" s="458"/>
-      <c r="D16" s="460"/>
-      <c r="E16" s="460"/>
+      <c r="A16" s="454"/>
+      <c r="B16" s="454"/>
+      <c r="C16" s="455"/>
+      <c r="D16" s="454"/>
+      <c r="E16" s="454"/>
       <c r="F16" s="307" t="s">
         <v>177</v>
       </c>
@@ -25001,11 +25075,11 @@
       <c r="Y16" s="73"/>
     </row>
     <row r="17" spans="1:50" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="460"/>
-      <c r="B17" s="460"/>
-      <c r="C17" s="458"/>
-      <c r="D17" s="460"/>
-      <c r="E17" s="460"/>
+      <c r="A17" s="454"/>
+      <c r="B17" s="454"/>
+      <c r="C17" s="455"/>
+      <c r="D17" s="454"/>
+      <c r="E17" s="454"/>
       <c r="F17" s="309" t="s">
         <v>180</v>
       </c>
@@ -25066,17 +25140,17 @@
       <c r="Y17" s="73"/>
     </row>
     <row r="18" spans="1:50" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="460"/>
-      <c r="B18" s="460" t="s">
+      <c r="A18" s="454"/>
+      <c r="B18" s="454" t="s">
         <v>167</v>
       </c>
-      <c r="C18" s="458" t="s">
+      <c r="C18" s="455" t="s">
         <v>188</v>
       </c>
-      <c r="D18" s="458" t="s">
+      <c r="D18" s="455" t="s">
         <v>189</v>
       </c>
-      <c r="E18" s="460" t="s">
+      <c r="E18" s="454" t="s">
         <v>193</v>
       </c>
       <c r="F18" s="315" t="s">
@@ -25085,7 +25159,7 @@
       <c r="G18" s="315" t="s">
         <v>80</v>
       </c>
-      <c r="H18" s="458" t="s">
+      <c r="H18" s="455" t="s">
         <v>194</v>
       </c>
       <c r="I18" s="362">
@@ -25155,18 +25229,18 @@
       <c r="Y18" s="73"/>
     </row>
     <row r="19" spans="1:50" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="460"/>
-      <c r="B19" s="460"/>
-      <c r="C19" s="458"/>
-      <c r="D19" s="458"/>
-      <c r="E19" s="460"/>
+      <c r="A19" s="454"/>
+      <c r="B19" s="454"/>
+      <c r="C19" s="455"/>
+      <c r="D19" s="455"/>
+      <c r="E19" s="454"/>
       <c r="F19" s="302" t="s">
         <v>173</v>
       </c>
       <c r="G19" s="302" t="s">
         <v>80</v>
       </c>
-      <c r="H19" s="458"/>
+      <c r="H19" s="455"/>
       <c r="I19" s="363">
         <f>I18</f>
         <v>0.52</v>
@@ -25234,13 +25308,13 @@
       <c r="Y19" s="73"/>
     </row>
     <row r="20" spans="1:50" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="460"/>
-      <c r="B20" s="460"/>
-      <c r="C20" s="458"/>
-      <c r="D20" s="460" t="s">
+      <c r="A20" s="454"/>
+      <c r="B20" s="454"/>
+      <c r="C20" s="455"/>
+      <c r="D20" s="454" t="s">
         <v>191</v>
       </c>
-      <c r="E20" s="460"/>
+      <c r="E20" s="454"/>
       <c r="F20" s="305" t="s">
         <v>175</v>
       </c>
@@ -25301,11 +25375,11 @@
       <c r="Y20" s="73"/>
     </row>
     <row r="21" spans="1:50" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="460"/>
-      <c r="B21" s="460"/>
-      <c r="C21" s="458"/>
-      <c r="D21" s="460"/>
-      <c r="E21" s="460"/>
+      <c r="A21" s="454"/>
+      <c r="B21" s="454"/>
+      <c r="C21" s="455"/>
+      <c r="D21" s="454"/>
+      <c r="E21" s="454"/>
       <c r="F21" s="307" t="s">
         <v>177</v>
       </c>
@@ -25366,11 +25440,11 @@
       <c r="Y21" s="73"/>
     </row>
     <row r="22" spans="1:50" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="460"/>
-      <c r="B22" s="460"/>
-      <c r="C22" s="458"/>
-      <c r="D22" s="460"/>
-      <c r="E22" s="460"/>
+      <c r="A22" s="454"/>
+      <c r="B22" s="454"/>
+      <c r="C22" s="455"/>
+      <c r="D22" s="454"/>
+      <c r="E22" s="454"/>
       <c r="F22" s="309" t="s">
         <v>180</v>
       </c>
@@ -25459,30 +25533,30 @@
     <row r="24" spans="1:50" ht="25.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="7"/>
-      <c r="C24" s="465" t="s">
+      <c r="C24" s="459" t="s">
         <v>196</v>
       </c>
-      <c r="D24" s="465"/>
-      <c r="E24" s="465"/>
-      <c r="F24" s="465"/>
-      <c r="G24" s="465"/>
-      <c r="H24" s="465"/>
-      <c r="I24" s="465"/>
-      <c r="J24" s="465"/>
-      <c r="K24" s="465"/>
-      <c r="L24" s="465"/>
-      <c r="M24" s="465"/>
-      <c r="N24" s="465"/>
-      <c r="O24" s="465"/>
-      <c r="P24" s="465"/>
-      <c r="Q24" s="465"/>
-      <c r="R24" s="465"/>
-      <c r="S24" s="465"/>
-      <c r="T24" s="465"/>
-      <c r="U24" s="465"/>
-      <c r="V24" s="465"/>
-      <c r="W24" s="465"/>
-      <c r="X24" s="465"/>
+      <c r="D24" s="459"/>
+      <c r="E24" s="459"/>
+      <c r="F24" s="459"/>
+      <c r="G24" s="459"/>
+      <c r="H24" s="459"/>
+      <c r="I24" s="459"/>
+      <c r="J24" s="459"/>
+      <c r="K24" s="459"/>
+      <c r="L24" s="459"/>
+      <c r="M24" s="459"/>
+      <c r="N24" s="459"/>
+      <c r="O24" s="459"/>
+      <c r="P24" s="459"/>
+      <c r="Q24" s="459"/>
+      <c r="R24" s="459"/>
+      <c r="S24" s="459"/>
+      <c r="T24" s="459"/>
+      <c r="U24" s="459"/>
+      <c r="V24" s="459"/>
+      <c r="W24" s="459"/>
+      <c r="X24" s="459"/>
     </row>
     <row r="25" spans="1:50" ht="43.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
@@ -25503,35 +25577,35 @@
       <c r="H25" s="63" t="s">
         <v>149</v>
       </c>
-      <c r="I25" s="466" t="s">
+      <c r="I25" s="460" t="s">
         <v>199</v>
       </c>
-      <c r="J25" s="467"/>
-      <c r="K25" s="467"/>
-      <c r="L25" s="467"/>
-      <c r="M25" s="467"/>
-      <c r="N25" s="467"/>
-      <c r="O25" s="467"/>
-      <c r="P25" s="467"/>
-      <c r="Q25" s="467"/>
-      <c r="R25" s="467"/>
-      <c r="S25" s="467"/>
-      <c r="T25" s="467"/>
-      <c r="U25" s="467"/>
-      <c r="V25" s="467"/>
-      <c r="W25" s="467"/>
-      <c r="X25" s="468"/>
+      <c r="J25" s="461"/>
+      <c r="K25" s="461"/>
+      <c r="L25" s="461"/>
+      <c r="M25" s="461"/>
+      <c r="N25" s="461"/>
+      <c r="O25" s="461"/>
+      <c r="P25" s="461"/>
+      <c r="Q25" s="461"/>
+      <c r="R25" s="461"/>
+      <c r="S25" s="461"/>
+      <c r="T25" s="461"/>
+      <c r="U25" s="461"/>
+      <c r="V25" s="461"/>
+      <c r="W25" s="461"/>
+      <c r="X25" s="462"/>
     </row>
     <row r="26" spans="1:50" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="84"/>
-      <c r="C26" s="462" t="s">
+      <c r="C26" s="456" t="s">
         <v>196</v>
       </c>
-      <c r="D26" s="462" t="s">
+      <c r="D26" s="456" t="s">
         <v>55</v>
       </c>
-      <c r="E26" s="462"/>
+      <c r="E26" s="456"/>
       <c r="F26" s="300" t="s">
         <v>171</v>
       </c>
@@ -25541,25 +25615,24 @@
       <c r="H26" s="64" t="s">
         <v>200</v>
       </c>
-      <c r="I26" s="455" t="e">
-        <f>(G26*0.112)*#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="J26" s="456"/>
-      <c r="K26" s="456"/>
-      <c r="L26" s="456"/>
-      <c r="M26" s="456"/>
-      <c r="N26" s="456"/>
-      <c r="O26" s="456"/>
-      <c r="P26" s="456"/>
-      <c r="Q26" s="456"/>
-      <c r="R26" s="456"/>
-      <c r="S26" s="456"/>
-      <c r="T26" s="456"/>
-      <c r="U26" s="456"/>
-      <c r="V26" s="456"/>
-      <c r="W26" s="456"/>
-      <c r="X26" s="457"/>
+      <c r="I26" s="598">
+        <v>0.46300000000000002</v>
+      </c>
+      <c r="J26" s="599"/>
+      <c r="K26" s="599"/>
+      <c r="L26" s="599"/>
+      <c r="M26" s="599"/>
+      <c r="N26" s="599"/>
+      <c r="O26" s="599"/>
+      <c r="P26" s="599"/>
+      <c r="Q26" s="599"/>
+      <c r="R26" s="599"/>
+      <c r="S26" s="599"/>
+      <c r="T26" s="599"/>
+      <c r="U26" s="599"/>
+      <c r="V26" s="599"/>
+      <c r="W26" s="599"/>
+      <c r="X26" s="602"/>
       <c r="Z26" s="351" t="s">
         <v>201</v>
       </c>
@@ -25571,9 +25644,9 @@
     <row r="27" spans="1:50" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
-      <c r="C27" s="463"/>
-      <c r="D27" s="463"/>
-      <c r="E27" s="463"/>
+      <c r="C27" s="457"/>
+      <c r="D27" s="457"/>
+      <c r="E27" s="457"/>
       <c r="F27" s="300" t="s">
         <v>173</v>
       </c>
@@ -25583,25 +25656,24 @@
       <c r="H27" s="64" t="s">
         <v>200</v>
       </c>
-      <c r="I27" s="455" t="e">
-        <f>(G27*0.112)*#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="J27" s="456"/>
-      <c r="K27" s="456"/>
-      <c r="L27" s="456"/>
-      <c r="M27" s="456"/>
-      <c r="N27" s="456"/>
-      <c r="O27" s="456"/>
-      <c r="P27" s="456"/>
-      <c r="Q27" s="456"/>
-      <c r="R27" s="456"/>
-      <c r="S27" s="456"/>
-      <c r="T27" s="456"/>
-      <c r="U27" s="456"/>
-      <c r="V27" s="456"/>
-      <c r="W27" s="456"/>
-      <c r="X27" s="457"/>
+      <c r="I27" s="600">
+        <v>0.46300000000000002</v>
+      </c>
+      <c r="J27" s="601"/>
+      <c r="K27" s="601"/>
+      <c r="L27" s="601"/>
+      <c r="M27" s="601"/>
+      <c r="N27" s="601"/>
+      <c r="O27" s="601"/>
+      <c r="P27" s="601"/>
+      <c r="Q27" s="601"/>
+      <c r="R27" s="601"/>
+      <c r="S27" s="601"/>
+      <c r="T27" s="601"/>
+      <c r="U27" s="601"/>
+      <c r="V27" s="601"/>
+      <c r="W27" s="601"/>
+      <c r="X27" s="603"/>
       <c r="Z27" s="351" t="s">
         <v>202</v>
       </c>
@@ -25613,9 +25685,9 @@
     <row r="28" spans="1:50" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="7"/>
-      <c r="C28" s="463"/>
-      <c r="D28" s="463"/>
-      <c r="E28" s="463"/>
+      <c r="C28" s="457"/>
+      <c r="D28" s="457"/>
+      <c r="E28" s="457"/>
       <c r="F28" s="300" t="s">
         <v>175</v>
       </c>
@@ -25625,25 +25697,24 @@
       <c r="H28" s="64" t="s">
         <v>200</v>
       </c>
-      <c r="I28" s="455" t="e">
-        <f>(G28*0.112)*#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="J28" s="456"/>
-      <c r="K28" s="456"/>
-      <c r="L28" s="456"/>
-      <c r="M28" s="456"/>
-      <c r="N28" s="456"/>
-      <c r="O28" s="456"/>
-      <c r="P28" s="456"/>
-      <c r="Q28" s="456"/>
-      <c r="R28" s="456"/>
-      <c r="S28" s="456"/>
-      <c r="T28" s="456"/>
-      <c r="U28" s="456"/>
-      <c r="V28" s="456"/>
-      <c r="W28" s="456"/>
-      <c r="X28" s="457"/>
+      <c r="I28" s="600">
+        <v>0.46300000000000002</v>
+      </c>
+      <c r="J28" s="601"/>
+      <c r="K28" s="601"/>
+      <c r="L28" s="601"/>
+      <c r="M28" s="601"/>
+      <c r="N28" s="601"/>
+      <c r="O28" s="601"/>
+      <c r="P28" s="601"/>
+      <c r="Q28" s="601"/>
+      <c r="R28" s="601"/>
+      <c r="S28" s="601"/>
+      <c r="T28" s="601"/>
+      <c r="U28" s="601"/>
+      <c r="V28" s="601"/>
+      <c r="W28" s="601"/>
+      <c r="X28" s="603"/>
       <c r="Y28" s="56"/>
       <c r="Z28" s="351" t="s">
         <v>203</v>
@@ -25652,36 +25723,36 @@
         <f>AA27</f>
         <v>6800</v>
       </c>
-      <c r="AB28" s="454"/>
-      <c r="AC28" s="454"/>
-      <c r="AD28" s="454"/>
-      <c r="AE28" s="454"/>
-      <c r="AF28" s="454"/>
-      <c r="AG28" s="454"/>
-      <c r="AH28" s="454"/>
-      <c r="AI28" s="454"/>
-      <c r="AJ28" s="454"/>
-      <c r="AK28" s="454"/>
-      <c r="AL28" s="454"/>
-      <c r="AM28" s="454"/>
-      <c r="AN28" s="454"/>
-      <c r="AO28" s="454"/>
-      <c r="AP28" s="454"/>
-      <c r="AQ28" s="454"/>
-      <c r="AR28" s="454"/>
-      <c r="AS28" s="454"/>
-      <c r="AT28" s="454"/>
-      <c r="AU28" s="454"/>
-      <c r="AV28" s="454"/>
-      <c r="AW28" s="454"/>
-      <c r="AX28" s="454"/>
+      <c r="AB28" s="465"/>
+      <c r="AC28" s="465"/>
+      <c r="AD28" s="465"/>
+      <c r="AE28" s="465"/>
+      <c r="AF28" s="465"/>
+      <c r="AG28" s="465"/>
+      <c r="AH28" s="465"/>
+      <c r="AI28" s="465"/>
+      <c r="AJ28" s="465"/>
+      <c r="AK28" s="465"/>
+      <c r="AL28" s="465"/>
+      <c r="AM28" s="465"/>
+      <c r="AN28" s="465"/>
+      <c r="AO28" s="465"/>
+      <c r="AP28" s="465"/>
+      <c r="AQ28" s="465"/>
+      <c r="AR28" s="465"/>
+      <c r="AS28" s="465"/>
+      <c r="AT28" s="465"/>
+      <c r="AU28" s="465"/>
+      <c r="AV28" s="465"/>
+      <c r="AW28" s="465"/>
+      <c r="AX28" s="465"/>
     </row>
     <row r="29" spans="1:50" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="7"/>
-      <c r="C29" s="463"/>
-      <c r="D29" s="463"/>
-      <c r="E29" s="463"/>
+      <c r="C29" s="457"/>
+      <c r="D29" s="457"/>
+      <c r="E29" s="457"/>
       <c r="F29" s="300" t="s">
         <v>177</v>
       </c>
@@ -25691,25 +25762,24 @@
       <c r="H29" s="301" t="s">
         <v>204</v>
       </c>
-      <c r="I29" s="455" t="e">
-        <f>(G29*0.112)*#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="J29" s="456"/>
-      <c r="K29" s="456"/>
-      <c r="L29" s="456"/>
-      <c r="M29" s="456"/>
-      <c r="N29" s="456"/>
-      <c r="O29" s="456"/>
-      <c r="P29" s="456"/>
-      <c r="Q29" s="456"/>
-      <c r="R29" s="456"/>
-      <c r="S29" s="456"/>
-      <c r="T29" s="456"/>
-      <c r="U29" s="456"/>
-      <c r="V29" s="456"/>
-      <c r="W29" s="456"/>
-      <c r="X29" s="457"/>
+      <c r="I29" s="600">
+        <v>0.42099999999999999</v>
+      </c>
+      <c r="J29" s="601"/>
+      <c r="K29" s="601"/>
+      <c r="L29" s="601"/>
+      <c r="M29" s="601"/>
+      <c r="N29" s="601"/>
+      <c r="O29" s="601"/>
+      <c r="P29" s="601"/>
+      <c r="Q29" s="601"/>
+      <c r="R29" s="601"/>
+      <c r="S29" s="601"/>
+      <c r="T29" s="601"/>
+      <c r="U29" s="601"/>
+      <c r="V29" s="601"/>
+      <c r="W29" s="601"/>
+      <c r="X29" s="603"/>
       <c r="Z29" s="351" t="s">
         <v>205</v>
       </c>
@@ -25721,9 +25791,9 @@
     <row r="30" spans="1:50" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="7"/>
-      <c r="C30" s="464"/>
-      <c r="D30" s="464"/>
-      <c r="E30" s="464"/>
+      <c r="C30" s="458"/>
+      <c r="D30" s="458"/>
+      <c r="E30" s="458"/>
       <c r="F30" s="300" t="s">
         <v>180</v>
       </c>
@@ -25733,25 +25803,24 @@
       <c r="H30" s="301" t="s">
         <v>207</v>
       </c>
-      <c r="I30" s="455" t="e">
-        <f>(0.6*0.112)*#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="J30" s="456"/>
-      <c r="K30" s="456"/>
-      <c r="L30" s="456"/>
-      <c r="M30" s="456"/>
-      <c r="N30" s="456"/>
-      <c r="O30" s="456"/>
-      <c r="P30" s="456"/>
-      <c r="Q30" s="456"/>
-      <c r="R30" s="456"/>
-      <c r="S30" s="456"/>
-      <c r="T30" s="456"/>
-      <c r="U30" s="456"/>
-      <c r="V30" s="456"/>
-      <c r="W30" s="456"/>
-      <c r="X30" s="457"/>
+      <c r="I30" s="600">
+        <v>0.252</v>
+      </c>
+      <c r="J30" s="601"/>
+      <c r="K30" s="601"/>
+      <c r="L30" s="601"/>
+      <c r="M30" s="601"/>
+      <c r="N30" s="601"/>
+      <c r="O30" s="601"/>
+      <c r="P30" s="601"/>
+      <c r="Q30" s="601"/>
+      <c r="R30" s="601"/>
+      <c r="S30" s="601"/>
+      <c r="T30" s="601"/>
+      <c r="U30" s="601"/>
+      <c r="V30" s="601"/>
+      <c r="W30" s="601"/>
+      <c r="X30" s="603"/>
     </row>
     <row r="31" spans="1:50" x14ac:dyDescent="0.25">
       <c r="E31" s="3" t="s">
@@ -25768,27 +25837,13 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="A13:A22"/>
-    <mergeCell ref="B13:B17"/>
-    <mergeCell ref="C13:C17"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E17"/>
-    <mergeCell ref="D15:D17"/>
-    <mergeCell ref="B18:B22"/>
-    <mergeCell ref="C18:C22"/>
-    <mergeCell ref="E18:E22"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="C26:C30"/>
-    <mergeCell ref="D26:D30"/>
-    <mergeCell ref="C24:X24"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="I25:X25"/>
-    <mergeCell ref="E26:E30"/>
-    <mergeCell ref="I26:X26"/>
-    <mergeCell ref="I27:X27"/>
-    <mergeCell ref="I28:X28"/>
+    <mergeCell ref="AL28:AP28"/>
+    <mergeCell ref="AQ28:AT28"/>
+    <mergeCell ref="AU28:AX28"/>
+    <mergeCell ref="I29:X29"/>
+    <mergeCell ref="I30:X30"/>
+    <mergeCell ref="AB28:AF28"/>
+    <mergeCell ref="AG28:AK28"/>
     <mergeCell ref="H8:H9"/>
     <mergeCell ref="A1:X1"/>
     <mergeCell ref="A3:A7"/>
@@ -25801,13 +25856,27 @@
     <mergeCell ref="C8:C12"/>
     <mergeCell ref="D8:D12"/>
     <mergeCell ref="E8:E12"/>
-    <mergeCell ref="AL28:AP28"/>
-    <mergeCell ref="AQ28:AT28"/>
-    <mergeCell ref="AU28:AX28"/>
-    <mergeCell ref="I29:X29"/>
-    <mergeCell ref="I30:X30"/>
-    <mergeCell ref="AB28:AF28"/>
-    <mergeCell ref="AG28:AK28"/>
+    <mergeCell ref="C26:C30"/>
+    <mergeCell ref="D26:D30"/>
+    <mergeCell ref="C24:X24"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="I25:X25"/>
+    <mergeCell ref="E26:E30"/>
+    <mergeCell ref="I26:X26"/>
+    <mergeCell ref="I27:X27"/>
+    <mergeCell ref="I28:X28"/>
+    <mergeCell ref="A13:A22"/>
+    <mergeCell ref="B13:B17"/>
+    <mergeCell ref="C13:C17"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E17"/>
+    <mergeCell ref="D15:D17"/>
+    <mergeCell ref="B18:B22"/>
+    <mergeCell ref="C18:C22"/>
+    <mergeCell ref="E18:E22"/>
+    <mergeCell ref="D18:D19"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H26" r:id="rId1" xr:uid="{DABFE6CB-B473-47DF-B585-2F887CAC1E59}"/>
@@ -25844,15 +25913,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="469" t="str">
+      <c r="A1" s="471" t="str">
         <f>"HVAC system - "&amp;Prototype!A2</f>
         <v>HVAC system - RetailStripMall</v>
       </c>
-      <c r="B1" s="469"/>
-      <c r="C1" s="469"/>
-      <c r="D1" s="469"/>
-      <c r="E1" s="469"/>
-      <c r="F1" s="469"/>
+      <c r="B1" s="471"/>
+      <c r="C1" s="471"/>
+      <c r="D1" s="471"/>
+      <c r="E1" s="471"/>
+      <c r="F1" s="471"/>
     </row>
     <row r="2" spans="1:10" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="326" t="s">
@@ -25917,10 +25986,10 @@
       <c r="F4" s="321" t="s">
         <v>225</v>
       </c>
-      <c r="G4" s="485"/>
-      <c r="H4" s="485"/>
-      <c r="I4" s="485"/>
-      <c r="J4" s="485"/>
+      <c r="G4" s="466"/>
+      <c r="H4" s="466"/>
+      <c r="I4" s="466"/>
+      <c r="J4" s="466"/>
     </row>
     <row r="5" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
@@ -25943,13 +26012,13 @@
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="483" t="s">
+      <c r="A8" s="482" t="s">
         <v>226</v>
       </c>
-      <c r="B8" s="484"/>
-      <c r="C8" s="484"/>
-      <c r="D8" s="484"/>
-      <c r="E8" s="484"/>
+      <c r="B8" s="483"/>
+      <c r="C8" s="483"/>
+      <c r="D8" s="483"/>
+      <c r="E8" s="483"/>
     </row>
     <row r="9" spans="1:10" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="66" t="s">
@@ -25972,16 +26041,16 @@
       <c r="A10" s="284" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="486">
+      <c r="B10" s="469">
         <v>2008</v>
       </c>
-      <c r="C10" s="479" t="s">
+      <c r="C10" s="470" t="s">
         <v>228</v>
       </c>
-      <c r="D10" s="471" t="s">
+      <c r="D10" s="467" t="s">
         <v>229</v>
       </c>
-      <c r="E10" s="471" t="s">
+      <c r="E10" s="467" t="s">
         <v>230</v>
       </c>
     </row>
@@ -25989,19 +26058,19 @@
       <c r="A11" s="284" t="s">
         <v>173</v>
       </c>
-      <c r="B11" s="486"/>
-      <c r="C11" s="479"/>
-      <c r="D11" s="481"/>
-      <c r="E11" s="481"/>
+      <c r="B11" s="469"/>
+      <c r="C11" s="470"/>
+      <c r="D11" s="468"/>
+      <c r="E11" s="468"/>
     </row>
     <row r="12" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="284" t="s">
         <v>175</v>
       </c>
-      <c r="B12" s="486"/>
-      <c r="C12" s="479"/>
-      <c r="D12" s="481"/>
-      <c r="E12" s="481"/>
+      <c r="B12" s="469"/>
+      <c r="C12" s="470"/>
+      <c r="D12" s="468"/>
+      <c r="E12" s="468"/>
     </row>
     <row r="13" spans="1:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="284" t="s">
@@ -26057,17 +26126,17 @@
       <c r="E17" s="369"/>
     </row>
     <row r="18" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="476" t="s">
+      <c r="A18" s="477" t="s">
         <v>237</v>
       </c>
-      <c r="B18" s="476"/>
-      <c r="C18" s="476"/>
-      <c r="D18" s="477"/>
-      <c r="E18" s="477"/>
-      <c r="F18" s="477"/>
-      <c r="G18" s="477"/>
-      <c r="H18" s="477"/>
-      <c r="I18" s="478"/>
+      <c r="B18" s="477"/>
+      <c r="C18" s="477"/>
+      <c r="D18" s="478"/>
+      <c r="E18" s="478"/>
+      <c r="F18" s="478"/>
+      <c r="G18" s="478"/>
+      <c r="H18" s="478"/>
+      <c r="I18" s="479"/>
     </row>
     <row r="19" spans="1:9" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="325" t="s">
@@ -26099,7 +26168,7 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="60.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="479" t="s">
+      <c r="A20" s="470" t="s">
         <v>179</v>
       </c>
       <c r="B20" s="480" t="s">
@@ -26111,20 +26180,20 @@
       <c r="D20" s="368">
         <v>2.5</v>
       </c>
-      <c r="E20" s="481">
+      <c r="E20" s="468">
         <v>0.65</v>
       </c>
-      <c r="F20" s="471" t="s">
+      <c r="F20" s="467" t="s">
         <v>247</v>
       </c>
-      <c r="G20" s="482"/>
-      <c r="H20" s="471" t="s">
+      <c r="G20" s="481"/>
+      <c r="H20" s="467" t="s">
         <v>248</v>
       </c>
       <c r="I20" s="298"/>
     </row>
     <row r="21" spans="1:9" ht="60.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="479"/>
+      <c r="A21" s="470"/>
       <c r="B21" s="480"/>
       <c r="C21" s="368" t="s">
         <v>249</v>
@@ -26132,10 +26201,10 @@
       <c r="D21" s="368">
         <v>4.09</v>
       </c>
-      <c r="E21" s="481"/>
-      <c r="F21" s="471"/>
-      <c r="G21" s="482"/>
-      <c r="H21" s="471"/>
+      <c r="E21" s="468"/>
+      <c r="F21" s="467"/>
+      <c r="G21" s="481"/>
+      <c r="H21" s="467"/>
       <c r="I21" s="298"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -26165,10 +26234,10 @@
       <c r="I23" s="297"/>
     </row>
     <row r="24" spans="1:9" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="473" t="s">
+      <c r="A24" s="474" t="s">
         <v>221</v>
       </c>
-      <c r="B24" s="475" t="s">
+      <c r="B24" s="476" t="s">
         <v>252</v>
       </c>
       <c r="C24" s="371" t="s">
@@ -26177,35 +26246,35 @@
       <c r="D24" s="372" t="s">
         <v>254</v>
       </c>
-      <c r="E24" s="471">
+      <c r="E24" s="467">
         <v>0.65</v>
       </c>
-      <c r="F24" s="471" t="s">
+      <c r="F24" s="467" t="s">
         <v>255</v>
       </c>
       <c r="G24" s="373">
         <v>0.74399999999999999</v>
       </c>
-      <c r="H24" s="471" t="s">
+      <c r="H24" s="467" t="s">
         <v>256</v>
       </c>
       <c r="I24" s="368"/>
     </row>
     <row r="25" spans="1:9" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="474"/>
-      <c r="B25" s="475"/>
+      <c r="A25" s="475"/>
+      <c r="B25" s="476"/>
       <c r="C25" s="374" t="s">
         <v>257</v>
       </c>
       <c r="D25" s="375" t="s">
         <v>254</v>
       </c>
-      <c r="E25" s="472"/>
-      <c r="F25" s="472"/>
+      <c r="E25" s="473"/>
+      <c r="F25" s="473"/>
       <c r="G25" s="376">
         <v>0.72</v>
       </c>
-      <c r="H25" s="472"/>
+      <c r="H25" s="473"/>
       <c r="I25" s="377"/>
     </row>
     <row r="26" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -26220,30 +26289,30 @@
       <c r="I26" s="369"/>
     </row>
     <row r="27" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="443" t="s">
+      <c r="A27" s="444" t="s">
         <v>258</v>
       </c>
-      <c r="B27" s="470"/>
-      <c r="C27" s="470"/>
-      <c r="D27" s="470"/>
-      <c r="E27" s="470"/>
-      <c r="F27" s="470"/>
-      <c r="G27" s="470"/>
-      <c r="H27" s="470"/>
-      <c r="I27" s="470"/>
+      <c r="B27" s="472"/>
+      <c r="C27" s="472"/>
+      <c r="D27" s="472"/>
+      <c r="E27" s="472"/>
+      <c r="F27" s="472"/>
+      <c r="G27" s="472"/>
+      <c r="H27" s="472"/>
+      <c r="I27" s="472"/>
     </row>
     <row r="28" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="443" t="s">
+      <c r="A28" s="444" t="s">
         <v>259</v>
       </c>
-      <c r="B28" s="443"/>
-      <c r="C28" s="443"/>
-      <c r="D28" s="443"/>
-      <c r="E28" s="443"/>
-      <c r="F28" s="443"/>
-      <c r="G28" s="443"/>
-      <c r="H28" s="443"/>
-      <c r="I28" s="443"/>
+      <c r="B28" s="444"/>
+      <c r="C28" s="444"/>
+      <c r="D28" s="444"/>
+      <c r="E28" s="444"/>
+      <c r="F28" s="444"/>
+      <c r="G28" s="444"/>
+      <c r="H28" s="444"/>
+      <c r="I28" s="444"/>
     </row>
     <row r="29" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="379"/>
@@ -26467,11 +26536,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="E10:E12"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A28:I28"/>
     <mergeCell ref="A27:I27"/>
@@ -26488,6 +26552,11 @@
     <mergeCell ref="G20:G21"/>
     <mergeCell ref="H20:H21"/>
     <mergeCell ref="A8:E8"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="E10:E12"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
@@ -26531,20 +26600,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="459" t="str">
+      <c r="A1" s="463" t="str">
         <f>"Outdoor Airflow Rate - "&amp;Prototype!A2</f>
         <v>Outdoor Airflow Rate - RetailStripMall</v>
       </c>
-      <c r="B1" s="459"/>
-      <c r="C1" s="459"/>
-      <c r="D1" s="459"/>
-      <c r="E1" s="459"/>
-      <c r="F1" s="459"/>
-      <c r="G1" s="459"/>
-      <c r="H1" s="459"/>
-      <c r="I1" s="459"/>
-      <c r="J1" s="459"/>
-      <c r="K1" s="459"/>
+      <c r="B1" s="463"/>
+      <c r="C1" s="463"/>
+      <c r="D1" s="463"/>
+      <c r="E1" s="463"/>
+      <c r="F1" s="463"/>
+      <c r="G1" s="463"/>
+      <c r="H1" s="463"/>
+      <c r="I1" s="463"/>
+      <c r="J1" s="463"/>
+      <c r="K1" s="463"/>
       <c r="L1" s="73"/>
     </row>
     <row r="2" spans="1:12" ht="47.4" customHeight="1" x14ac:dyDescent="0.25">
@@ -26796,27 +26865,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="459" t="str">
+      <c r="A1" s="463" t="str">
         <f>"Thermostat Setpoints - "&amp;Prototype!A2</f>
         <v>Thermostat Setpoints - RetailStripMall</v>
       </c>
-      <c r="B1" s="459"/>
-      <c r="C1" s="459"/>
-      <c r="D1" s="459"/>
-      <c r="E1" s="459"/>
-      <c r="F1" s="459"/>
-      <c r="G1" s="459"/>
-      <c r="H1" s="459"/>
-      <c r="I1" s="459"/>
-      <c r="J1" s="459"/>
-      <c r="K1" s="459"/>
-      <c r="L1" s="459"/>
-      <c r="M1" s="459"/>
-      <c r="N1" s="459"/>
-      <c r="O1" s="459"/>
-      <c r="P1" s="459"/>
-      <c r="Q1" s="459"/>
-      <c r="R1" s="459"/>
+      <c r="B1" s="463"/>
+      <c r="C1" s="463"/>
+      <c r="D1" s="463"/>
+      <c r="E1" s="463"/>
+      <c r="F1" s="463"/>
+      <c r="G1" s="463"/>
+      <c r="H1" s="463"/>
+      <c r="I1" s="463"/>
+      <c r="J1" s="463"/>
+      <c r="K1" s="463"/>
+      <c r="L1" s="463"/>
+      <c r="M1" s="463"/>
+      <c r="N1" s="463"/>
+      <c r="O1" s="463"/>
+      <c r="P1" s="463"/>
+      <c r="Q1" s="463"/>
+      <c r="R1" s="463"/>
     </row>
     <row r="2" spans="1:18" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="65" t="s">
@@ -26926,7 +26995,7 @@
       <c r="Q3" s="284">
         <v>70</v>
       </c>
-      <c r="R3" s="487" t="s">
+      <c r="R3" s="484" t="s">
         <v>272</v>
       </c>
     </row>
@@ -26982,7 +27051,7 @@
       <c r="Q4" s="284">
         <v>60</v>
       </c>
-      <c r="R4" s="488"/>
+      <c r="R4" s="485"/>
     </row>
     <row r="5" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="284" t="s">
@@ -27036,7 +27105,7 @@
       <c r="Q5" s="284">
         <v>75</v>
       </c>
-      <c r="R5" s="488"/>
+      <c r="R5" s="485"/>
     </row>
     <row r="6" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="284" t="s">
@@ -27090,7 +27159,7 @@
       <c r="Q6" s="284">
         <v>85</v>
       </c>
-      <c r="R6" s="489"/>
+      <c r="R6" s="486"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -27135,16 +27204,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="491" t="str">
+      <c r="A1" s="488" t="str">
         <f>"Water Heater - "&amp;Prototype!A2</f>
         <v>Water Heater - RetailStripMall</v>
       </c>
-      <c r="B1" s="469"/>
-      <c r="C1" s="469"/>
-      <c r="D1" s="469"/>
-      <c r="E1" s="469"/>
-      <c r="F1" s="469"/>
-      <c r="G1" s="469"/>
+      <c r="B1" s="471"/>
+      <c r="C1" s="471"/>
+      <c r="D1" s="471"/>
+      <c r="E1" s="471"/>
+      <c r="F1" s="471"/>
+      <c r="G1" s="471"/>
     </row>
     <row r="2" spans="1:10" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="219" t="s">
@@ -27225,16 +27294,16 @@
       <c r="D5" s="317"/>
     </row>
     <row r="6" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="500" t="s">
+      <c r="A6" s="497" t="s">
         <v>285</v>
       </c>
-      <c r="B6" s="459"/>
-      <c r="C6" s="459"/>
-      <c r="D6" s="459"/>
-      <c r="E6" s="459"/>
-      <c r="F6" s="459"/>
-      <c r="G6" s="459"/>
-      <c r="H6" s="459"/>
+      <c r="B6" s="463"/>
+      <c r="C6" s="463"/>
+      <c r="D6" s="463"/>
+      <c r="E6" s="463"/>
+      <c r="F6" s="463"/>
+      <c r="G6" s="463"/>
+      <c r="H6" s="463"/>
     </row>
     <row r="7" spans="1:10" ht="61.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="129" t="s">
@@ -27289,7 +27358,7 @@
         <f>F8/60</f>
         <v>0.19125196884989998</v>
       </c>
-      <c r="H8" s="501" t="s">
+      <c r="H8" s="498" t="s">
         <v>292</v>
       </c>
     </row>
@@ -27320,7 +27389,7 @@
         <f t="shared" ref="G9:G11" si="1">F9/60</f>
         <v>9.5623239627899995E-2</v>
       </c>
-      <c r="H9" s="502"/>
+      <c r="H9" s="499"/>
     </row>
     <row r="10" spans="1:10" ht="28.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="131" t="str">
@@ -27349,7 +27418,7 @@
         <f t="shared" si="1"/>
         <v>9.5623239627899995E-2</v>
       </c>
-      <c r="H10" s="502"/>
+      <c r="H10" s="499"/>
     </row>
     <row r="11" spans="1:10" s="4" customFormat="1" ht="28.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="133" t="str">
@@ -27378,18 +27447,18 @@
         <f t="shared" si="1"/>
         <v>9.5623239627899995E-2</v>
       </c>
-      <c r="H11" s="503"/>
+      <c r="H11" s="500"/>
     </row>
     <row r="12" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="252" t="s">
         <v>293</v>
       </c>
-      <c r="B12" s="504" t="s">
+      <c r="B12" s="501" t="s">
         <v>294</v>
       </c>
-      <c r="C12" s="505"/>
-      <c r="D12" s="505"/>
-      <c r="E12" s="506"/>
+      <c r="C12" s="502"/>
+      <c r="D12" s="502"/>
+      <c r="E12" s="503"/>
       <c r="F12" s="283">
         <f>_xlfn.LET(
   _xlpm.g,SUMIF($B$8:$B$11,"Gas*",$F$8:$F$11),
@@ -27398,7 +27467,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="253"/>
-      <c r="H12" s="507" t="s">
+      <c r="H12" s="504" t="s">
         <v>295</v>
       </c>
     </row>
@@ -27406,12 +27475,12 @@
       <c r="A13" s="252" t="s">
         <v>296</v>
       </c>
-      <c r="B13" s="504" t="s">
+      <c r="B13" s="501" t="s">
         <v>297</v>
       </c>
-      <c r="C13" s="505"/>
-      <c r="D13" s="505"/>
-      <c r="E13" s="506"/>
+      <c r="C13" s="502"/>
+      <c r="D13" s="502"/>
+      <c r="E13" s="503"/>
       <c r="F13" s="283">
         <f>_xlfn.LET(
   _xlpm.g,SUMIF($B$8:$B$11,"Gas*",$F$8:$F$11),
@@ -27420,7 +27489,7 @@
         <v>75</v>
       </c>
       <c r="G13" s="253"/>
-      <c r="H13" s="508"/>
+      <c r="H13" s="505"/>
     </row>
     <row r="14" spans="1:10" s="254" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14"/>
@@ -27527,19 +27596,19 @@
       <c r="G20" s="258"/>
     </row>
     <row r="21" spans="1:12" s="254" customFormat="1" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="492" t="s">
+      <c r="A21" s="489" t="s">
         <v>305</v>
       </c>
-      <c r="B21" s="493"/>
-      <c r="C21" s="493"/>
-      <c r="D21" s="493"/>
-      <c r="E21" s="493"/>
-      <c r="F21" s="493"/>
-      <c r="G21" s="493"/>
-      <c r="H21" s="493"/>
-      <c r="I21" s="493"/>
-      <c r="J21" s="493"/>
-      <c r="K21" s="493"/>
+      <c r="B21" s="490"/>
+      <c r="C21" s="490"/>
+      <c r="D21" s="490"/>
+      <c r="E21" s="490"/>
+      <c r="F21" s="490"/>
+      <c r="G21" s="490"/>
+      <c r="H21" s="490"/>
+      <c r="I21" s="490"/>
+      <c r="J21" s="490"/>
+      <c r="K21" s="490"/>
     </row>
     <row r="22" spans="1:12" s="254" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="390" t="s">
@@ -27560,14 +27629,14 @@
       <c r="F22" s="390" t="s">
         <v>311</v>
       </c>
-      <c r="G22" s="494" t="s">
+      <c r="G22" s="491" t="s">
         <v>312</v>
       </c>
-      <c r="H22" s="495"/>
-      <c r="I22" s="496" t="s">
+      <c r="H22" s="492"/>
+      <c r="I22" s="493" t="s">
         <v>313</v>
       </c>
-      <c r="J22" s="496"/>
+      <c r="J22" s="493"/>
       <c r="K22" s="391" t="s">
         <v>314</v>
       </c>
@@ -27611,7 +27680,7 @@
       <c r="J23" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K23" s="497" t="s">
+      <c r="K23" s="494" t="s">
         <v>317</v>
       </c>
     </row>
@@ -27653,7 +27722,7 @@
       <c r="J24" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K24" s="498"/>
+      <c r="K24" s="495"/>
     </row>
     <row r="25" spans="1:12" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="392" t="s">
@@ -27693,7 +27762,7 @@
       <c r="J25" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K25" s="498"/>
+      <c r="K25" s="495"/>
     </row>
     <row r="26" spans="1:12" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="392" t="s">
@@ -27733,7 +27802,7 @@
       <c r="J26" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K26" s="498"/>
+      <c r="K26" s="495"/>
     </row>
     <row r="27" spans="1:12" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="392" t="s">
@@ -27773,7 +27842,7 @@
       <c r="J27" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K27" s="498"/>
+      <c r="K27" s="495"/>
     </row>
     <row r="28" spans="1:12" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="392" t="s">
@@ -27813,7 +27882,7 @@
       <c r="J28" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K28" s="498"/>
+      <c r="K28" s="495"/>
     </row>
     <row r="29" spans="1:12" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="392" t="s">
@@ -27853,7 +27922,7 @@
       <c r="J29" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K29" s="498"/>
+      <c r="K29" s="495"/>
     </row>
     <row r="30" spans="1:12" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="392" t="s">
@@ -27893,7 +27962,7 @@
       <c r="J30" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K30" s="498"/>
+      <c r="K30" s="495"/>
     </row>
     <row r="31" spans="1:12" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="392" t="s">
@@ -27933,7 +28002,7 @@
       <c r="J31" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K31" s="498"/>
+      <c r="K31" s="495"/>
     </row>
     <row r="32" spans="1:12" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="392" t="s">
@@ -27973,7 +28042,7 @@
       <c r="J32" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K32" s="498"/>
+      <c r="K32" s="495"/>
     </row>
     <row r="33" spans="1:11" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="392" t="s">
@@ -28013,7 +28082,7 @@
       <c r="J33" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K33" s="498"/>
+      <c r="K33" s="495"/>
     </row>
     <row r="34" spans="1:11" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="392" t="s">
@@ -28053,7 +28122,7 @@
       <c r="J34" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K34" s="498"/>
+      <c r="K34" s="495"/>
     </row>
     <row r="35" spans="1:11" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="392" t="s">
@@ -28093,7 +28162,7 @@
       <c r="J35" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K35" s="498"/>
+      <c r="K35" s="495"/>
     </row>
     <row r="36" spans="1:11" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="392" t="s">
@@ -28133,7 +28202,7 @@
       <c r="J36" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K36" s="498"/>
+      <c r="K36" s="495"/>
     </row>
     <row r="37" spans="1:11" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="392" t="s">
@@ -28173,7 +28242,7 @@
       <c r="J37" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K37" s="498"/>
+      <c r="K37" s="495"/>
     </row>
     <row r="38" spans="1:11" s="254" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="392" t="s">
@@ -28213,7 +28282,7 @@
       <c r="J38" s="397" t="s">
         <v>316</v>
       </c>
-      <c r="K38" s="499"/>
+      <c r="K38" s="496"/>
     </row>
     <row r="39" spans="1:11" s="254" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C39" s="258"/>
@@ -28234,16 +28303,16 @@
       <c r="G41" s="258"/>
     </row>
     <row r="42" spans="1:11" s="254" customFormat="1" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="490" t="s">
+      <c r="A42" s="487" t="s">
         <v>326</v>
       </c>
-      <c r="B42" s="459"/>
-      <c r="C42" s="459"/>
-      <c r="D42" s="459"/>
-      <c r="E42" s="459"/>
-      <c r="F42" s="459"/>
-      <c r="G42" s="459"/>
-      <c r="H42" s="459"/>
+      <c r="B42" s="463"/>
+      <c r="C42" s="463"/>
+      <c r="D42" s="463"/>
+      <c r="E42" s="463"/>
+      <c r="F42" s="463"/>
+      <c r="G42" s="463"/>
+      <c r="H42" s="463"/>
     </row>
     <row r="43" spans="1:11" s="259" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A43" s="398" t="s">
@@ -28944,38 +29013,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="511" t="str">
+      <c r="A1" s="508" t="str">
         <f>"Interior Lighting - "&amp;Prototype!A2</f>
         <v>Interior Lighting - RetailStripMall</v>
       </c>
-      <c r="B1" s="512"/>
-      <c r="C1" s="512"/>
-      <c r="D1" s="512"/>
-      <c r="E1" s="512"/>
-      <c r="F1" s="512"/>
-      <c r="G1" s="512"/>
-      <c r="H1" s="513"/>
+      <c r="B1" s="509"/>
+      <c r="C1" s="509"/>
+      <c r="D1" s="509"/>
+      <c r="E1" s="509"/>
+      <c r="F1" s="509"/>
+      <c r="G1" s="509"/>
+      <c r="H1" s="510"/>
     </row>
     <row r="2" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="509" t="s">
+      <c r="A2" s="506" t="s">
         <v>338</v>
       </c>
-      <c r="B2" s="510" t="s">
+      <c r="B2" s="507" t="s">
         <v>339</v>
       </c>
-      <c r="C2" s="510"/>
-      <c r="D2" s="510"/>
-      <c r="E2" s="510" t="s">
+      <c r="C2" s="507"/>
+      <c r="D2" s="507"/>
+      <c r="E2" s="507" t="s">
         <v>179</v>
       </c>
-      <c r="F2" s="510"/>
-      <c r="G2" s="510"/>
-      <c r="H2" s="514" t="s">
+      <c r="F2" s="507"/>
+      <c r="G2" s="507"/>
+      <c r="H2" s="511" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="32.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="509"/>
+      <c r="A3" s="506"/>
       <c r="B3" s="323" t="s">
         <v>340</v>
       </c>
@@ -28994,7 +29063,7 @@
       <c r="G3" s="323" t="s">
         <v>214</v>
       </c>
-      <c r="H3" s="515"/>
+      <c r="H3" s="512"/>
     </row>
     <row r="4" spans="1:8" ht="47.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="263" t="str">
@@ -29102,6 +29171,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003D1D6A7EB2452B4A86A9506D4E13D4C9" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7cd6ed0cd056f112062446d0d1c544ce">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="41613948-0554-4f13-babe-277410c056ca" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="60ca449bf2be89171a15d05d28af00ea" ns2:_="">
     <xsd:import namespace="41613948-0554-4f13-babe-277410c056ca"/>
@@ -29239,22 +29323,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20816333-575B-4274-8A3E-18699B071E90}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7921AF10-0BF8-441A-BDBA-64AF3E09D45F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8883227C-5317-464B-AEF8-1C96313FD89F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -29270,21 +29356,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7921AF10-0BF8-441A-BDBA-64AF3E09D45F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20816333-575B-4274-8A3E-18699B071E90}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>